<commit_message>
Add grid and network costs
</commit_message>
<xml_diff>
--- a/VT_IE_SRV.xlsx
+++ b/VT_IE_SRV.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model-VAv2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5D510CB-B01A-4A23-8BA5-465746C8CBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257292A9-ACDF-4184-9080-C1B466285B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="83" r:id="rId1"/>
@@ -1384,7 +1384,7 @@
     <author>Alessandro Chiodi</author>
   </authors>
   <commentList>
-    <comment ref="I4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+    <comment ref="N4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1627,7 +1627,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
+    <comment ref="T4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1720,7 +1720,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
+    <comment ref="U4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
       <text>
         <r>
           <rPr>
@@ -1735,7 +1735,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
+    <comment ref="V4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
       <text>
         <r>
           <rPr>
@@ -4426,7 +4426,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="628">
   <si>
     <t>Unit</t>
   </si>
@@ -6455,6 +6455,18 @@
   <si>
     <t>Last Updated : 1st September 2022</t>
   </si>
+  <si>
+    <t>INVCOST</t>
+  </si>
+  <si>
+    <t>FIXOM</t>
+  </si>
+  <si>
+    <t>LIFE</t>
+  </si>
+  <si>
+    <t>CAP2ACT</t>
+  </si>
 </sst>
 </file>
 
@@ -6469,7 +6481,7 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="76">
+  <fonts count="78">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7017,8 +7029,21 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="47">
+  <fills count="48">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7282,6 +7307,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="43"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="173">
     <border>
@@ -9464,7 +9495,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="133">
+  <cellStyleXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -9598,8 +9629,11 @@
     <xf numFmtId="0" fontId="75" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="624">
+  <cellXfs count="625">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -11342,6 +11376,9 @@
     <xf numFmtId="38" fontId="34" fillId="0" borderId="156" xfId="128" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="76" fillId="47" borderId="0" xfId="130" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="127" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -11402,7 +11439,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="133">
+  <cellStyles count="136">
     <cellStyle name="20 % - Akzent1" xfId="49" hidden="1" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="20 % - Akzent1" xfId="74" hidden="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="20 % - Akzent1" xfId="115" hidden="1" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
@@ -11519,12 +11556,15 @@
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Hyperlink" xfId="43" builtinId="8"/>
+    <cellStyle name="Hyperlink 2" xfId="135" xr:uid="{5DF4E031-1A26-443C-89CC-DA1BA500A4A7}"/>
+    <cellStyle name="Hyperlink 3" xfId="133" xr:uid="{FC6B72DE-D8B9-42FC-9D35-B9EC58B45E22}"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="127" xr:uid="{C8015E5B-BB2C-4455-8316-ECA2C120BAAB}"/>
     <cellStyle name="Normal 2 2" xfId="130" xr:uid="{1AA6CE7F-ECFC-47CF-9235-BD9996F92AF5}"/>
+    <cellStyle name="Normal 3" xfId="134" xr:uid="{D9A83FE8-2EC2-4FAF-98ED-A285F82DFE25}"/>
     <cellStyle name="Normal_1990 and 1998 CIP - Prices Quantity and CO2(MH)" xfId="129" xr:uid="{04DF7896-4666-4107-A97C-3E460D392FBF}"/>
     <cellStyle name="Normal_2000balx" xfId="128" xr:uid="{B3C00B14-B312-4A46-9ED8-30E2DAAA08A1}"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
@@ -11943,7 +11983,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>28575</xdr:colOff>
+          <xdr:colOff>31750</xdr:colOff>
           <xdr:row>3</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -12460,17 +12500,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E413D879-EF52-4D62-9DB2-77F8A9CE34B4}">
   <sheetPr codeName="Sheet17"/>
   <dimension ref="A1:Z99"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" customWidth="1"/>
-    <col min="8" max="10" width="8.140625" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" customWidth="1"/>
-    <col min="12" max="12" width="8.140625" customWidth="1"/>
+    <col min="1" max="4" width="21.7265625" customWidth="1"/>
+    <col min="5" max="6" width="14.1796875" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" customWidth="1"/>
+    <col min="8" max="10" width="8.1796875" customWidth="1"/>
+    <col min="11" max="11" width="9.7265625" customWidth="1"/>
+    <col min="12" max="12" width="8.1796875" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" customWidth="1"/>
-    <col min="15" max="15" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -12894,12 +12934,12 @@
       <c r="Z15" s="308"/>
     </row>
     <row r="16" spans="1:26" ht="102.75" customHeight="1">
-      <c r="A16" s="604" t="s">
+      <c r="A16" s="605" t="s">
         <v>591</v>
       </c>
-      <c r="B16" s="604"/>
-      <c r="C16" s="604"/>
-      <c r="D16" s="604"/>
+      <c r="B16" s="605"/>
+      <c r="C16" s="605"/>
+      <c r="D16" s="605"/>
       <c r="E16" s="309"/>
       <c r="F16" s="309"/>
       <c r="G16" s="310"/>
@@ -12983,11 +13023,11 @@
       <c r="A19" s="314" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="603" t="s">
+      <c r="B19" s="604" t="s">
         <v>603</v>
       </c>
-      <c r="C19" s="603"/>
-      <c r="D19" s="603"/>
+      <c r="C19" s="604"/>
+      <c r="D19" s="604"/>
       <c r="E19" s="315"/>
       <c r="F19" s="315"/>
       <c r="G19" s="316"/>
@@ -13015,11 +13055,11 @@
       <c r="A20" s="314" t="s">
         <v>592</v>
       </c>
-      <c r="B20" s="603" t="s">
+      <c r="B20" s="604" t="s">
         <v>604</v>
       </c>
-      <c r="C20" s="603"/>
-      <c r="D20" s="603"/>
+      <c r="C20" s="604"/>
+      <c r="D20" s="604"/>
       <c r="E20" s="315"/>
       <c r="F20" s="315"/>
       <c r="G20" s="316"/>
@@ -13107,9 +13147,9 @@
       <c r="A23" s="314" t="s">
         <v>594</v>
       </c>
-      <c r="B23" s="603"/>
-      <c r="C23" s="603"/>
-      <c r="D23" s="603"/>
+      <c r="B23" s="604"/>
+      <c r="C23" s="604"/>
+      <c r="D23" s="604"/>
       <c r="E23" s="308"/>
       <c r="F23" s="308"/>
       <c r="G23" s="308"/>
@@ -13193,11 +13233,11 @@
       <c r="A26" s="314" t="s">
         <v>595</v>
       </c>
-      <c r="B26" s="603" t="s">
+      <c r="B26" s="604" t="s">
         <v>602</v>
       </c>
-      <c r="C26" s="603"/>
-      <c r="D26" s="603"/>
+      <c r="C26" s="604"/>
+      <c r="D26" s="604"/>
       <c r="E26" s="308"/>
       <c r="F26" s="308"/>
       <c r="G26" s="308"/>
@@ -13313,11 +13353,11 @@
       <c r="A30" s="314" t="s">
         <v>597</v>
       </c>
-      <c r="B30" s="605" t="s">
+      <c r="B30" s="606" t="s">
         <v>598</v>
       </c>
-      <c r="C30" s="603"/>
-      <c r="D30" s="603"/>
+      <c r="C30" s="604"/>
+      <c r="D30" s="604"/>
       <c r="E30" s="319"/>
       <c r="F30" s="319"/>
       <c r="G30" s="308"/>
@@ -13345,11 +13385,11 @@
       <c r="A31" s="314" t="s">
         <v>599</v>
       </c>
-      <c r="B31" s="603" t="s">
+      <c r="B31" s="604" t="s">
         <v>600</v>
       </c>
-      <c r="C31" s="603"/>
-      <c r="D31" s="603"/>
+      <c r="C31" s="604"/>
+      <c r="D31" s="604"/>
       <c r="E31" s="319"/>
       <c r="F31" s="319"/>
       <c r="G31" s="308"/>
@@ -15305,37 +15345,37 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:AD21"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="2.28515625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="2.26953125" style="9" customWidth="1"/>
     <col min="2" max="2" width="22" style="9" customWidth="1"/>
-    <col min="3" max="3" width="48.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="48.7265625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" style="9" customWidth="1"/>
     <col min="6" max="10" width="13" style="9" customWidth="1"/>
-    <col min="11" max="11" width="4.85546875" style="9" customWidth="1"/>
-    <col min="12" max="13" width="14.5703125" style="9" customWidth="1"/>
-    <col min="14" max="14" width="16.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="44.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="9.7109375" style="9" customWidth="1"/>
-    <col min="21" max="21" width="4.85546875" style="9" customWidth="1"/>
-    <col min="22" max="22" width="21.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="16.7109375" style="9" customWidth="1"/>
-    <col min="31" max="31" width="4.85546875" style="9" customWidth="1"/>
-    <col min="32" max="32" width="8.85546875" style="9"/>
-    <col min="33" max="34" width="19.28515625" style="9" customWidth="1"/>
-    <col min="35" max="48" width="8.85546875" style="9"/>
-    <col min="49" max="49" width="12.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="50" max="16384" width="8.85546875" style="9"/>
+    <col min="11" max="11" width="4.81640625" style="9" customWidth="1"/>
+    <col min="12" max="13" width="14.54296875" style="9" customWidth="1"/>
+    <col min="14" max="14" width="16.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="44.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="20" width="9.7265625" style="9" customWidth="1"/>
+    <col min="21" max="21" width="4.81640625" style="9" customWidth="1"/>
+    <col min="22" max="22" width="21.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="29" max="30" width="16.7265625" style="9" customWidth="1"/>
+    <col min="31" max="31" width="4.81640625" style="9" customWidth="1"/>
+    <col min="32" max="32" width="8.81640625" style="9"/>
+    <col min="33" max="34" width="19.26953125" style="9" customWidth="1"/>
+    <col min="35" max="48" width="8.81640625" style="9"/>
+    <col min="49" max="49" width="12.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="50" max="16384" width="8.81640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:30" ht="23.25">
+    <row r="1" spans="2:30" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>504</v>
       </c>
@@ -15358,7 +15398,7 @@
       <c r="T2" s="36"/>
       <c r="AD2" s="14"/>
     </row>
-    <row r="3" spans="2:30" ht="15.75" thickBot="1">
+    <row r="3" spans="2:30" ht="15" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>4</v>
       </c>
@@ -15413,25 +15453,25 @@
       <c r="T3" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="V3" s="608" t="s">
+      <c r="V3" s="609" t="s">
         <v>378</v>
       </c>
-      <c r="W3" s="608" t="s">
+      <c r="W3" s="609" t="s">
         <v>160</v>
       </c>
-      <c r="X3" s="608" t="s">
+      <c r="X3" s="609" t="s">
         <v>81</v>
       </c>
-      <c r="Y3" s="608" t="s">
+      <c r="Y3" s="609" t="s">
         <v>498</v>
       </c>
-      <c r="Z3" s="608" t="s">
+      <c r="Z3" s="609" t="s">
         <v>499</v>
       </c>
-      <c r="AA3" s="608" t="s">
+      <c r="AA3" s="609" t="s">
         <v>500</v>
       </c>
-      <c r="AB3" s="608" t="s">
+      <c r="AB3" s="609" t="s">
         <v>501</v>
       </c>
       <c r="AC3" s="49" t="s">
@@ -15439,7 +15479,7 @@
       </c>
       <c r="AD3" s="135"/>
     </row>
-    <row r="4" spans="2:30" ht="51.75" thickBot="1">
+    <row r="4" spans="2:30" ht="52.5" thickBot="1">
       <c r="B4" s="39" t="s">
         <v>125</v>
       </c>
@@ -15494,13 +15534,13 @@
       <c r="T4" s="39" t="s">
         <v>121</v>
       </c>
-      <c r="V4" s="609"/>
-      <c r="W4" s="609"/>
-      <c r="X4" s="609"/>
-      <c r="Y4" s="609"/>
-      <c r="Z4" s="609"/>
-      <c r="AA4" s="609"/>
-      <c r="AB4" s="609"/>
+      <c r="V4" s="610"/>
+      <c r="W4" s="610"/>
+      <c r="X4" s="610"/>
+      <c r="Y4" s="610"/>
+      <c r="Z4" s="610"/>
+      <c r="AA4" s="610"/>
+      <c r="AB4" s="610"/>
       <c r="AC4" s="13" t="s">
         <v>146</v>
       </c>
@@ -16547,37 +16587,37 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:AD13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="2.28515625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="2.26953125" style="9" customWidth="1"/>
     <col min="2" max="2" width="22" style="9" customWidth="1"/>
-    <col min="3" max="3" width="51.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="51.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" style="9" customWidth="1"/>
     <col min="6" max="10" width="13" style="9" customWidth="1"/>
-    <col min="11" max="11" width="4.85546875" style="9" customWidth="1"/>
-    <col min="12" max="13" width="12.42578125" style="9" customWidth="1"/>
-    <col min="14" max="14" width="17.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="51.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="10.85546875" style="9" customWidth="1"/>
-    <col min="21" max="21" width="4.85546875" style="9" customWidth="1"/>
-    <col min="22" max="22" width="21.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="16.7109375" style="9" customWidth="1"/>
-    <col min="31" max="31" width="4.85546875" style="9" customWidth="1"/>
-    <col min="32" max="32" width="8.85546875" style="9"/>
-    <col min="33" max="34" width="19.28515625" style="9" customWidth="1"/>
-    <col min="35" max="48" width="8.85546875" style="9"/>
-    <col min="49" max="49" width="12.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="50" max="16384" width="8.85546875" style="9"/>
+    <col min="11" max="11" width="4.81640625" style="9" customWidth="1"/>
+    <col min="12" max="13" width="12.453125" style="9" customWidth="1"/>
+    <col min="14" max="14" width="17.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="51.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="20" width="10.81640625" style="9" customWidth="1"/>
+    <col min="21" max="21" width="4.81640625" style="9" customWidth="1"/>
+    <col min="22" max="22" width="21.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="29" max="30" width="16.7265625" style="9" customWidth="1"/>
+    <col min="31" max="31" width="4.81640625" style="9" customWidth="1"/>
+    <col min="32" max="32" width="8.81640625" style="9"/>
+    <col min="33" max="34" width="19.26953125" style="9" customWidth="1"/>
+    <col min="35" max="48" width="8.81640625" style="9"/>
+    <col min="49" max="49" width="12.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="50" max="16384" width="8.81640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:30" ht="23.25">
+    <row r="1" spans="2:30" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>91</v>
       </c>
@@ -16600,7 +16640,7 @@
       <c r="T2" s="36"/>
       <c r="AD2" s="14"/>
     </row>
-    <row r="3" spans="2:30" ht="15.75" thickBot="1">
+    <row r="3" spans="2:30" ht="15" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>4</v>
       </c>
@@ -16655,25 +16695,25 @@
       <c r="T3" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="V3" s="608" t="s">
+      <c r="V3" s="609" t="s">
         <v>378</v>
       </c>
-      <c r="W3" s="608" t="s">
+      <c r="W3" s="609" t="s">
         <v>160</v>
       </c>
-      <c r="X3" s="608" t="s">
+      <c r="X3" s="609" t="s">
         <v>81</v>
       </c>
-      <c r="Y3" s="608" t="s">
+      <c r="Y3" s="609" t="s">
         <v>498</v>
       </c>
-      <c r="Z3" s="608" t="s">
+      <c r="Z3" s="609" t="s">
         <v>499</v>
       </c>
-      <c r="AA3" s="608" t="s">
+      <c r="AA3" s="609" t="s">
         <v>500</v>
       </c>
-      <c r="AB3" s="608" t="s">
+      <c r="AB3" s="609" t="s">
         <v>501</v>
       </c>
       <c r="AC3" s="49" t="s">
@@ -16681,7 +16721,7 @@
       </c>
       <c r="AD3" s="135"/>
     </row>
-    <row r="4" spans="2:30" ht="51.75" thickBot="1">
+    <row r="4" spans="2:30" ht="52.5" thickBot="1">
       <c r="B4" s="39" t="s">
         <v>125</v>
       </c>
@@ -16736,13 +16776,13 @@
       <c r="T4" s="39" t="s">
         <v>121</v>
       </c>
-      <c r="V4" s="609"/>
-      <c r="W4" s="609"/>
-      <c r="X4" s="609"/>
-      <c r="Y4" s="609"/>
-      <c r="Z4" s="609"/>
-      <c r="AA4" s="609"/>
-      <c r="AB4" s="609"/>
+      <c r="V4" s="610"/>
+      <c r="W4" s="610"/>
+      <c r="X4" s="610"/>
+      <c r="Y4" s="610"/>
+      <c r="Z4" s="610"/>
+      <c r="AA4" s="610"/>
+      <c r="AB4" s="610"/>
       <c r="AC4" s="13" t="s">
         <v>146</v>
       </c>
@@ -16750,7 +16790,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="5" spans="2:30" ht="25.5">
+    <row r="5" spans="2:30" ht="26">
       <c r="B5" s="42" t="s">
         <v>131</v>
       </c>
@@ -17464,37 +17504,37 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:AD19"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="2.28515625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="2.26953125" style="9" customWidth="1"/>
     <col min="2" max="2" width="22" style="9" customWidth="1"/>
-    <col min="3" max="3" width="51.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="51.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" style="9" customWidth="1"/>
     <col min="6" max="10" width="13" style="9" customWidth="1"/>
-    <col min="11" max="11" width="4.85546875" style="9" customWidth="1"/>
-    <col min="12" max="13" width="17.28515625" style="9" customWidth="1"/>
-    <col min="14" max="14" width="17.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="51.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="10.85546875" style="9" customWidth="1"/>
-    <col min="21" max="21" width="4.85546875" style="9" customWidth="1"/>
-    <col min="22" max="22" width="21.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="20.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="16.7109375" style="9" customWidth="1"/>
-    <col min="31" max="31" width="4.85546875" style="9" customWidth="1"/>
-    <col min="32" max="32" width="8.85546875" style="9"/>
-    <col min="33" max="34" width="19.28515625" style="9" customWidth="1"/>
-    <col min="35" max="48" width="8.85546875" style="9"/>
-    <col min="49" max="49" width="12.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="50" max="16384" width="8.85546875" style="9"/>
+    <col min="11" max="11" width="4.81640625" style="9" customWidth="1"/>
+    <col min="12" max="13" width="17.26953125" style="9" customWidth="1"/>
+    <col min="14" max="14" width="17.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="51.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="20" width="10.81640625" style="9" customWidth="1"/>
+    <col min="21" max="21" width="4.81640625" style="9" customWidth="1"/>
+    <col min="22" max="22" width="21.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="29" max="30" width="16.7265625" style="9" customWidth="1"/>
+    <col min="31" max="31" width="4.81640625" style="9" customWidth="1"/>
+    <col min="32" max="32" width="8.81640625" style="9"/>
+    <col min="33" max="34" width="19.26953125" style="9" customWidth="1"/>
+    <col min="35" max="48" width="8.81640625" style="9"/>
+    <col min="49" max="49" width="12.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="50" max="16384" width="8.81640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:30" ht="23.25">
+    <row r="1" spans="2:30" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>515</v>
       </c>
@@ -17517,7 +17557,7 @@
       <c r="T2" s="36"/>
       <c r="AD2" s="14"/>
     </row>
-    <row r="3" spans="2:30" ht="15.75" thickBot="1">
+    <row r="3" spans="2:30" ht="15" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>4</v>
       </c>
@@ -17572,25 +17612,25 @@
       <c r="T3" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="V3" s="608" t="s">
+      <c r="V3" s="609" t="s">
         <v>378</v>
       </c>
-      <c r="W3" s="608" t="s">
+      <c r="W3" s="609" t="s">
         <v>160</v>
       </c>
-      <c r="X3" s="608" t="s">
+      <c r="X3" s="609" t="s">
         <v>81</v>
       </c>
-      <c r="Y3" s="608" t="s">
+      <c r="Y3" s="609" t="s">
         <v>498</v>
       </c>
-      <c r="Z3" s="608" t="s">
+      <c r="Z3" s="609" t="s">
         <v>499</v>
       </c>
-      <c r="AA3" s="608" t="s">
+      <c r="AA3" s="609" t="s">
         <v>500</v>
       </c>
-      <c r="AB3" s="608" t="s">
+      <c r="AB3" s="609" t="s">
         <v>501</v>
       </c>
       <c r="AC3" s="49" t="s">
@@ -17598,7 +17638,7 @@
       </c>
       <c r="AD3" s="135"/>
     </row>
-    <row r="4" spans="2:30" ht="51.75" thickBot="1">
+    <row r="4" spans="2:30" ht="52.5" thickBot="1">
       <c r="B4" s="39" t="s">
         <v>125</v>
       </c>
@@ -17653,13 +17693,13 @@
       <c r="T4" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="V4" s="609"/>
-      <c r="W4" s="609"/>
-      <c r="X4" s="609"/>
-      <c r="Y4" s="609"/>
-      <c r="Z4" s="609"/>
-      <c r="AA4" s="609"/>
-      <c r="AB4" s="609"/>
+      <c r="V4" s="610"/>
+      <c r="W4" s="610"/>
+      <c r="X4" s="610"/>
+      <c r="Y4" s="610"/>
+      <c r="Z4" s="610"/>
+      <c r="AA4" s="610"/>
+      <c r="AB4" s="610"/>
       <c r="AC4" s="13" t="s">
         <v>146</v>
       </c>
@@ -18191,7 +18231,7 @@
         <v>0.48000000000000004</v>
       </c>
     </row>
-    <row r="14" spans="2:30" ht="23.25">
+    <row r="14" spans="2:30" ht="23.5">
       <c r="B14" s="47" t="s">
         <v>519</v>
       </c>
@@ -18201,7 +18241,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="2:30" ht="15.75" thickBot="1">
+    <row r="16" spans="2:30" ht="15" thickBot="1">
       <c r="B16" s="21" t="s">
         <v>520</v>
       </c>
@@ -18215,7 +18255,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="25.5">
+    <row r="17" spans="2:5" ht="26">
       <c r="B17" s="39" t="s">
         <v>606</v>
       </c>
@@ -18277,38 +18317,38 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:AD16"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="2.28515625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="2.26953125" style="9" customWidth="1"/>
     <col min="2" max="2" width="22" style="9" customWidth="1"/>
     <col min="3" max="3" width="36" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" style="9" customWidth="1"/>
     <col min="6" max="10" width="13" style="9" customWidth="1"/>
-    <col min="11" max="11" width="4.85546875" style="9" customWidth="1"/>
-    <col min="12" max="12" width="20.5703125" style="9" customWidth="1"/>
-    <col min="13" max="13" width="12.42578125" style="9" customWidth="1"/>
-    <col min="14" max="14" width="16.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="51.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="10.85546875" style="9" customWidth="1"/>
-    <col min="21" max="21" width="4.85546875" style="9" customWidth="1"/>
-    <col min="22" max="22" width="21.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="16.7109375" style="9" customWidth="1"/>
-    <col min="31" max="31" width="4.85546875" style="9" customWidth="1"/>
-    <col min="32" max="32" width="8.85546875" style="9"/>
-    <col min="33" max="34" width="19.28515625" style="9" customWidth="1"/>
-    <col min="35" max="48" width="8.85546875" style="9"/>
-    <col min="49" max="49" width="12.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="50" max="16384" width="8.85546875" style="9"/>
+    <col min="11" max="11" width="4.81640625" style="9" customWidth="1"/>
+    <col min="12" max="12" width="20.54296875" style="9" customWidth="1"/>
+    <col min="13" max="13" width="12.453125" style="9" customWidth="1"/>
+    <col min="14" max="14" width="16.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="51.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="20" width="10.81640625" style="9" customWidth="1"/>
+    <col min="21" max="21" width="4.81640625" style="9" customWidth="1"/>
+    <col min="22" max="22" width="21.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="29" max="30" width="16.7265625" style="9" customWidth="1"/>
+    <col min="31" max="31" width="4.81640625" style="9" customWidth="1"/>
+    <col min="32" max="32" width="8.81640625" style="9"/>
+    <col min="33" max="34" width="19.26953125" style="9" customWidth="1"/>
+    <col min="35" max="48" width="8.81640625" style="9"/>
+    <col min="49" max="49" width="12.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="50" max="16384" width="8.81640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:30" ht="23.25">
+    <row r="1" spans="2:30" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>516</v>
       </c>
@@ -18331,7 +18371,7 @@
       <c r="T2" s="36"/>
       <c r="AD2" s="14"/>
     </row>
-    <row r="3" spans="2:30" ht="15.75" thickBot="1">
+    <row r="3" spans="2:30" ht="15" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>4</v>
       </c>
@@ -18386,25 +18426,25 @@
       <c r="T3" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="V3" s="608" t="s">
+      <c r="V3" s="609" t="s">
         <v>378</v>
       </c>
-      <c r="W3" s="608" t="s">
+      <c r="W3" s="609" t="s">
         <v>160</v>
       </c>
-      <c r="X3" s="608" t="s">
+      <c r="X3" s="609" t="s">
         <v>81</v>
       </c>
-      <c r="Y3" s="608" t="s">
+      <c r="Y3" s="609" t="s">
         <v>498</v>
       </c>
-      <c r="Z3" s="608" t="s">
+      <c r="Z3" s="609" t="s">
         <v>499</v>
       </c>
-      <c r="AA3" s="608" t="s">
+      <c r="AA3" s="609" t="s">
         <v>500</v>
       </c>
-      <c r="AB3" s="608" t="s">
+      <c r="AB3" s="609" t="s">
         <v>501</v>
       </c>
       <c r="AC3" s="49" t="s">
@@ -18412,7 +18452,7 @@
       </c>
       <c r="AD3" s="135"/>
     </row>
-    <row r="4" spans="2:30" ht="51.75" thickBot="1">
+    <row r="4" spans="2:30" ht="52.5" thickBot="1">
       <c r="B4" s="39" t="s">
         <v>125</v>
       </c>
@@ -18467,13 +18507,13 @@
       <c r="T4" s="39" t="s">
         <v>121</v>
       </c>
-      <c r="V4" s="609"/>
-      <c r="W4" s="609"/>
-      <c r="X4" s="609"/>
-      <c r="Y4" s="609"/>
-      <c r="Z4" s="609"/>
-      <c r="AA4" s="609"/>
-      <c r="AB4" s="609"/>
+      <c r="V4" s="610"/>
+      <c r="W4" s="610"/>
+      <c r="X4" s="610"/>
+      <c r="Y4" s="610"/>
+      <c r="Z4" s="610"/>
+      <c r="AA4" s="610"/>
+      <c r="AB4" s="610"/>
       <c r="AC4" s="13" t="s">
         <v>146</v>
       </c>
@@ -18714,7 +18754,7 @@
         <v>5.6291760000000002</v>
       </c>
     </row>
-    <row r="11" spans="2:30" ht="23.25">
+    <row r="11" spans="2:30" ht="23.5">
       <c r="B11" s="47" t="s">
         <v>519</v>
       </c>
@@ -18724,7 +18764,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="2:30" ht="15.75" thickBot="1">
+    <row r="13" spans="2:30" ht="15" thickBot="1">
       <c r="B13" s="21" t="s">
         <v>520</v>
       </c>
@@ -18738,7 +18778,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="14" spans="2:30" ht="25.5">
+    <row r="14" spans="2:30" ht="26">
       <c r="B14" s="39" t="s">
         <v>606</v>
       </c>
@@ -18799,15 +18839,15 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:H19"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="2.42578125" style="9" customWidth="1"/>
-    <col min="2" max="8" width="14.85546875" style="9" customWidth="1"/>
-    <col min="9" max="19" width="11.28515625" style="9" customWidth="1"/>
-    <col min="20" max="16384" width="8.85546875" style="9"/>
+    <col min="1" max="1" width="2.453125" style="9" customWidth="1"/>
+    <col min="2" max="8" width="14.81640625" style="9" customWidth="1"/>
+    <col min="9" max="19" width="11.26953125" style="9" customWidth="1"/>
+    <col min="20" max="16384" width="8.81640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="23.25">
+    <row r="1" spans="2:8" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>78</v>
       </c>
@@ -18817,7 +18857,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="15.75" thickBot="1">
+    <row r="3" spans="2:8" ht="15" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>7</v>
       </c>
@@ -18846,7 +18886,7 @@
         <v>SRVSOL</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="25.5">
+    <row r="4" spans="2:8" ht="26">
       <c r="B4" s="39" t="s">
         <v>150</v>
       </c>
@@ -18959,7 +18999,7 @@
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
     </row>
-    <row r="16" spans="2:8" ht="15.75" thickBot="1">
+    <row r="16" spans="2:8" ht="15" thickBot="1">
       <c r="B16" s="12" t="s">
         <v>151</v>
       </c>
@@ -19006,46 +19046,46 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AS80"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="38.140625" style="85" customWidth="1"/>
+    <col min="1" max="1" width="38.1796875" style="85" customWidth="1"/>
     <col min="2" max="2" width="13" style="79" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="7.5703125" style="84" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="84"/>
-    <col min="6" max="6" width="6.140625" style="86" customWidth="1"/>
-    <col min="7" max="7" width="5.85546875" style="86" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.42578125" style="84" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.140625" style="86" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="7.54296875" style="84" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" style="84"/>
+    <col min="6" max="6" width="6.1796875" style="86" customWidth="1"/>
+    <col min="7" max="7" width="5.81640625" style="86" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.453125" style="84" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.1796875" style="86" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6" style="86" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.85546875" style="86" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" style="83" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.140625" style="79" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.140625" style="79" customWidth="1"/>
-    <col min="15" max="15" width="5.28515625" style="79" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="79" customWidth="1"/>
-    <col min="17" max="17" width="7.42578125" style="79" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.140625" style="79" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.28515625" style="79" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.42578125" style="79" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.42578125" style="79" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.85546875" style="79" bestFit="1" customWidth="1"/>
-    <col min="23" max="25" width="5.42578125" style="79" customWidth="1"/>
-    <col min="26" max="26" width="5.42578125" style="86" customWidth="1"/>
-    <col min="27" max="27" width="8.140625" style="83" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="6.7109375" style="83" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="5.5703125" style="79" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" style="79" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="8.7109375" style="79" customWidth="1"/>
-    <col min="33" max="33" width="5.5703125" style="79" customWidth="1"/>
-    <col min="34" max="34" width="5.85546875" style="79" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.81640625" style="86" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" style="83" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.1796875" style="79" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.1796875" style="79" customWidth="1"/>
+    <col min="15" max="15" width="5.26953125" style="79" customWidth="1"/>
+    <col min="16" max="16" width="7.453125" style="79" customWidth="1"/>
+    <col min="17" max="17" width="7.453125" style="79" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.1796875" style="79" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.26953125" style="79" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.453125" style="79" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.453125" style="79" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.81640625" style="79" bestFit="1" customWidth="1"/>
+    <col min="23" max="25" width="5.453125" style="79" customWidth="1"/>
+    <col min="26" max="26" width="5.453125" style="86" customWidth="1"/>
+    <col min="27" max="27" width="8.1796875" style="83" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="6.7265625" style="83" bestFit="1" customWidth="1"/>
+    <col min="29" max="30" width="5.54296875" style="79" customWidth="1"/>
+    <col min="31" max="31" width="8.7265625" style="79" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.7265625" style="79" customWidth="1"/>
+    <col min="33" max="33" width="5.54296875" style="79" customWidth="1"/>
+    <col min="34" max="34" width="5.81640625" style="79" bestFit="1" customWidth="1"/>
     <col min="35" max="37" width="7" style="79" customWidth="1"/>
-    <col min="38" max="40" width="5.5703125" style="79" customWidth="1"/>
-    <col min="41" max="41" width="8.7109375" style="83" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="4.42578125" style="83" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="9.28515625" style="79" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="9.140625" style="79"/>
-    <col min="45" max="45" width="9.140625" style="81"/>
-    <col min="46" max="16384" width="9.140625" style="79"/>
+    <col min="38" max="40" width="5.54296875" style="79" customWidth="1"/>
+    <col min="41" max="41" width="8.7265625" style="83" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="4.453125" style="83" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="9.26953125" style="79" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="9.1796875" style="79"/>
+    <col min="45" max="45" width="9.1796875" style="81"/>
+    <col min="46" max="16384" width="9.1796875" style="79"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="105.75" customHeight="1" thickBot="1">
@@ -25472,7 +25512,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.59055118110236227" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.19685039370078741"/>
-  <pageSetup paperSize="9" scale="41" fitToHeight="0" orientation="landscape" cellComments="asDisplayed" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="40" fitToHeight="0" orientation="landscape" cellComments="asDisplayed" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader>&amp;C&amp;"Myriad Pro,Regular"&amp;14Ireland's Energy Balance &amp;A</oddHeader>
     <oddFooter>&amp;L&amp;G&amp;RPage &amp;P of &amp;N</oddFooter>
@@ -25491,218 +25531,218 @@
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" style="202" customWidth="1"/>
-    <col min="2" max="15" width="13.7109375" style="188" customWidth="1"/>
-    <col min="16" max="241" width="9.140625" style="188"/>
+    <col min="2" max="15" width="13.7265625" style="188" customWidth="1"/>
+    <col min="16" max="241" width="9.1796875" style="188"/>
     <col min="242" max="242" width="18" style="188" customWidth="1"/>
-    <col min="243" max="256" width="13.7109375" style="188" customWidth="1"/>
-    <col min="257" max="497" width="9.140625" style="188"/>
+    <col min="243" max="256" width="13.7265625" style="188" customWidth="1"/>
+    <col min="257" max="497" width="9.1796875" style="188"/>
     <col min="498" max="498" width="18" style="188" customWidth="1"/>
-    <col min="499" max="512" width="13.7109375" style="188" customWidth="1"/>
-    <col min="513" max="753" width="9.140625" style="188"/>
+    <col min="499" max="512" width="13.7265625" style="188" customWidth="1"/>
+    <col min="513" max="753" width="9.1796875" style="188"/>
     <col min="754" max="754" width="18" style="188" customWidth="1"/>
-    <col min="755" max="768" width="13.7109375" style="188" customWidth="1"/>
-    <col min="769" max="1009" width="9.140625" style="188"/>
+    <col min="755" max="768" width="13.7265625" style="188" customWidth="1"/>
+    <col min="769" max="1009" width="9.1796875" style="188"/>
     <col min="1010" max="1010" width="18" style="188" customWidth="1"/>
-    <col min="1011" max="1024" width="13.7109375" style="188" customWidth="1"/>
-    <col min="1025" max="1265" width="9.140625" style="188"/>
+    <col min="1011" max="1024" width="13.7265625" style="188" customWidth="1"/>
+    <col min="1025" max="1265" width="9.1796875" style="188"/>
     <col min="1266" max="1266" width="18" style="188" customWidth="1"/>
-    <col min="1267" max="1280" width="13.7109375" style="188" customWidth="1"/>
-    <col min="1281" max="1521" width="9.140625" style="188"/>
+    <col min="1267" max="1280" width="13.7265625" style="188" customWidth="1"/>
+    <col min="1281" max="1521" width="9.1796875" style="188"/>
     <col min="1522" max="1522" width="18" style="188" customWidth="1"/>
-    <col min="1523" max="1536" width="13.7109375" style="188" customWidth="1"/>
-    <col min="1537" max="1777" width="9.140625" style="188"/>
+    <col min="1523" max="1536" width="13.7265625" style="188" customWidth="1"/>
+    <col min="1537" max="1777" width="9.1796875" style="188"/>
     <col min="1778" max="1778" width="18" style="188" customWidth="1"/>
-    <col min="1779" max="1792" width="13.7109375" style="188" customWidth="1"/>
-    <col min="1793" max="2033" width="9.140625" style="188"/>
+    <col min="1779" max="1792" width="13.7265625" style="188" customWidth="1"/>
+    <col min="1793" max="2033" width="9.1796875" style="188"/>
     <col min="2034" max="2034" width="18" style="188" customWidth="1"/>
-    <col min="2035" max="2048" width="13.7109375" style="188" customWidth="1"/>
-    <col min="2049" max="2289" width="9.140625" style="188"/>
+    <col min="2035" max="2048" width="13.7265625" style="188" customWidth="1"/>
+    <col min="2049" max="2289" width="9.1796875" style="188"/>
     <col min="2290" max="2290" width="18" style="188" customWidth="1"/>
-    <col min="2291" max="2304" width="13.7109375" style="188" customWidth="1"/>
-    <col min="2305" max="2545" width="9.140625" style="188"/>
+    <col min="2291" max="2304" width="13.7265625" style="188" customWidth="1"/>
+    <col min="2305" max="2545" width="9.1796875" style="188"/>
     <col min="2546" max="2546" width="18" style="188" customWidth="1"/>
-    <col min="2547" max="2560" width="13.7109375" style="188" customWidth="1"/>
-    <col min="2561" max="2801" width="9.140625" style="188"/>
+    <col min="2547" max="2560" width="13.7265625" style="188" customWidth="1"/>
+    <col min="2561" max="2801" width="9.1796875" style="188"/>
     <col min="2802" max="2802" width="18" style="188" customWidth="1"/>
-    <col min="2803" max="2816" width="13.7109375" style="188" customWidth="1"/>
-    <col min="2817" max="3057" width="9.140625" style="188"/>
+    <col min="2803" max="2816" width="13.7265625" style="188" customWidth="1"/>
+    <col min="2817" max="3057" width="9.1796875" style="188"/>
     <col min="3058" max="3058" width="18" style="188" customWidth="1"/>
-    <col min="3059" max="3072" width="13.7109375" style="188" customWidth="1"/>
-    <col min="3073" max="3313" width="9.140625" style="188"/>
+    <col min="3059" max="3072" width="13.7265625" style="188" customWidth="1"/>
+    <col min="3073" max="3313" width="9.1796875" style="188"/>
     <col min="3314" max="3314" width="18" style="188" customWidth="1"/>
-    <col min="3315" max="3328" width="13.7109375" style="188" customWidth="1"/>
-    <col min="3329" max="3569" width="9.140625" style="188"/>
+    <col min="3315" max="3328" width="13.7265625" style="188" customWidth="1"/>
+    <col min="3329" max="3569" width="9.1796875" style="188"/>
     <col min="3570" max="3570" width="18" style="188" customWidth="1"/>
-    <col min="3571" max="3584" width="13.7109375" style="188" customWidth="1"/>
-    <col min="3585" max="3825" width="9.140625" style="188"/>
+    <col min="3571" max="3584" width="13.7265625" style="188" customWidth="1"/>
+    <col min="3585" max="3825" width="9.1796875" style="188"/>
     <col min="3826" max="3826" width="18" style="188" customWidth="1"/>
-    <col min="3827" max="3840" width="13.7109375" style="188" customWidth="1"/>
-    <col min="3841" max="4081" width="9.140625" style="188"/>
+    <col min="3827" max="3840" width="13.7265625" style="188" customWidth="1"/>
+    <col min="3841" max="4081" width="9.1796875" style="188"/>
     <col min="4082" max="4082" width="18" style="188" customWidth="1"/>
-    <col min="4083" max="4096" width="13.7109375" style="188" customWidth="1"/>
-    <col min="4097" max="4337" width="9.140625" style="188"/>
+    <col min="4083" max="4096" width="13.7265625" style="188" customWidth="1"/>
+    <col min="4097" max="4337" width="9.1796875" style="188"/>
     <col min="4338" max="4338" width="18" style="188" customWidth="1"/>
-    <col min="4339" max="4352" width="13.7109375" style="188" customWidth="1"/>
-    <col min="4353" max="4593" width="9.140625" style="188"/>
+    <col min="4339" max="4352" width="13.7265625" style="188" customWidth="1"/>
+    <col min="4353" max="4593" width="9.1796875" style="188"/>
     <col min="4594" max="4594" width="18" style="188" customWidth="1"/>
-    <col min="4595" max="4608" width="13.7109375" style="188" customWidth="1"/>
-    <col min="4609" max="4849" width="9.140625" style="188"/>
+    <col min="4595" max="4608" width="13.7265625" style="188" customWidth="1"/>
+    <col min="4609" max="4849" width="9.1796875" style="188"/>
     <col min="4850" max="4850" width="18" style="188" customWidth="1"/>
-    <col min="4851" max="4864" width="13.7109375" style="188" customWidth="1"/>
-    <col min="4865" max="5105" width="9.140625" style="188"/>
+    <col min="4851" max="4864" width="13.7265625" style="188" customWidth="1"/>
+    <col min="4865" max="5105" width="9.1796875" style="188"/>
     <col min="5106" max="5106" width="18" style="188" customWidth="1"/>
-    <col min="5107" max="5120" width="13.7109375" style="188" customWidth="1"/>
-    <col min="5121" max="5361" width="9.140625" style="188"/>
+    <col min="5107" max="5120" width="13.7265625" style="188" customWidth="1"/>
+    <col min="5121" max="5361" width="9.1796875" style="188"/>
     <col min="5362" max="5362" width="18" style="188" customWidth="1"/>
-    <col min="5363" max="5376" width="13.7109375" style="188" customWidth="1"/>
-    <col min="5377" max="5617" width="9.140625" style="188"/>
+    <col min="5363" max="5376" width="13.7265625" style="188" customWidth="1"/>
+    <col min="5377" max="5617" width="9.1796875" style="188"/>
     <col min="5618" max="5618" width="18" style="188" customWidth="1"/>
-    <col min="5619" max="5632" width="13.7109375" style="188" customWidth="1"/>
-    <col min="5633" max="5873" width="9.140625" style="188"/>
+    <col min="5619" max="5632" width="13.7265625" style="188" customWidth="1"/>
+    <col min="5633" max="5873" width="9.1796875" style="188"/>
     <col min="5874" max="5874" width="18" style="188" customWidth="1"/>
-    <col min="5875" max="5888" width="13.7109375" style="188" customWidth="1"/>
-    <col min="5889" max="6129" width="9.140625" style="188"/>
+    <col min="5875" max="5888" width="13.7265625" style="188" customWidth="1"/>
+    <col min="5889" max="6129" width="9.1796875" style="188"/>
     <col min="6130" max="6130" width="18" style="188" customWidth="1"/>
-    <col min="6131" max="6144" width="13.7109375" style="188" customWidth="1"/>
-    <col min="6145" max="6385" width="9.140625" style="188"/>
+    <col min="6131" max="6144" width="13.7265625" style="188" customWidth="1"/>
+    <col min="6145" max="6385" width="9.1796875" style="188"/>
     <col min="6386" max="6386" width="18" style="188" customWidth="1"/>
-    <col min="6387" max="6400" width="13.7109375" style="188" customWidth="1"/>
-    <col min="6401" max="6641" width="9.140625" style="188"/>
+    <col min="6387" max="6400" width="13.7265625" style="188" customWidth="1"/>
+    <col min="6401" max="6641" width="9.1796875" style="188"/>
     <col min="6642" max="6642" width="18" style="188" customWidth="1"/>
-    <col min="6643" max="6656" width="13.7109375" style="188" customWidth="1"/>
-    <col min="6657" max="6897" width="9.140625" style="188"/>
+    <col min="6643" max="6656" width="13.7265625" style="188" customWidth="1"/>
+    <col min="6657" max="6897" width="9.1796875" style="188"/>
     <col min="6898" max="6898" width="18" style="188" customWidth="1"/>
-    <col min="6899" max="6912" width="13.7109375" style="188" customWidth="1"/>
-    <col min="6913" max="7153" width="9.140625" style="188"/>
+    <col min="6899" max="6912" width="13.7265625" style="188" customWidth="1"/>
+    <col min="6913" max="7153" width="9.1796875" style="188"/>
     <col min="7154" max="7154" width="18" style="188" customWidth="1"/>
-    <col min="7155" max="7168" width="13.7109375" style="188" customWidth="1"/>
-    <col min="7169" max="7409" width="9.140625" style="188"/>
+    <col min="7155" max="7168" width="13.7265625" style="188" customWidth="1"/>
+    <col min="7169" max="7409" width="9.1796875" style="188"/>
     <col min="7410" max="7410" width="18" style="188" customWidth="1"/>
-    <col min="7411" max="7424" width="13.7109375" style="188" customWidth="1"/>
-    <col min="7425" max="7665" width="9.140625" style="188"/>
+    <col min="7411" max="7424" width="13.7265625" style="188" customWidth="1"/>
+    <col min="7425" max="7665" width="9.1796875" style="188"/>
     <col min="7666" max="7666" width="18" style="188" customWidth="1"/>
-    <col min="7667" max="7680" width="13.7109375" style="188" customWidth="1"/>
-    <col min="7681" max="7921" width="9.140625" style="188"/>
+    <col min="7667" max="7680" width="13.7265625" style="188" customWidth="1"/>
+    <col min="7681" max="7921" width="9.1796875" style="188"/>
     <col min="7922" max="7922" width="18" style="188" customWidth="1"/>
-    <col min="7923" max="7936" width="13.7109375" style="188" customWidth="1"/>
-    <col min="7937" max="8177" width="9.140625" style="188"/>
+    <col min="7923" max="7936" width="13.7265625" style="188" customWidth="1"/>
+    <col min="7937" max="8177" width="9.1796875" style="188"/>
     <col min="8178" max="8178" width="18" style="188" customWidth="1"/>
-    <col min="8179" max="8192" width="13.7109375" style="188" customWidth="1"/>
-    <col min="8193" max="8433" width="9.140625" style="188"/>
+    <col min="8179" max="8192" width="13.7265625" style="188" customWidth="1"/>
+    <col min="8193" max="8433" width="9.1796875" style="188"/>
     <col min="8434" max="8434" width="18" style="188" customWidth="1"/>
-    <col min="8435" max="8448" width="13.7109375" style="188" customWidth="1"/>
-    <col min="8449" max="8689" width="9.140625" style="188"/>
+    <col min="8435" max="8448" width="13.7265625" style="188" customWidth="1"/>
+    <col min="8449" max="8689" width="9.1796875" style="188"/>
     <col min="8690" max="8690" width="18" style="188" customWidth="1"/>
-    <col min="8691" max="8704" width="13.7109375" style="188" customWidth="1"/>
-    <col min="8705" max="8945" width="9.140625" style="188"/>
+    <col min="8691" max="8704" width="13.7265625" style="188" customWidth="1"/>
+    <col min="8705" max="8945" width="9.1796875" style="188"/>
     <col min="8946" max="8946" width="18" style="188" customWidth="1"/>
-    <col min="8947" max="8960" width="13.7109375" style="188" customWidth="1"/>
-    <col min="8961" max="9201" width="9.140625" style="188"/>
+    <col min="8947" max="8960" width="13.7265625" style="188" customWidth="1"/>
+    <col min="8961" max="9201" width="9.1796875" style="188"/>
     <col min="9202" max="9202" width="18" style="188" customWidth="1"/>
-    <col min="9203" max="9216" width="13.7109375" style="188" customWidth="1"/>
-    <col min="9217" max="9457" width="9.140625" style="188"/>
+    <col min="9203" max="9216" width="13.7265625" style="188" customWidth="1"/>
+    <col min="9217" max="9457" width="9.1796875" style="188"/>
     <col min="9458" max="9458" width="18" style="188" customWidth="1"/>
-    <col min="9459" max="9472" width="13.7109375" style="188" customWidth="1"/>
-    <col min="9473" max="9713" width="9.140625" style="188"/>
+    <col min="9459" max="9472" width="13.7265625" style="188" customWidth="1"/>
+    <col min="9473" max="9713" width="9.1796875" style="188"/>
     <col min="9714" max="9714" width="18" style="188" customWidth="1"/>
-    <col min="9715" max="9728" width="13.7109375" style="188" customWidth="1"/>
-    <col min="9729" max="9969" width="9.140625" style="188"/>
+    <col min="9715" max="9728" width="13.7265625" style="188" customWidth="1"/>
+    <col min="9729" max="9969" width="9.1796875" style="188"/>
     <col min="9970" max="9970" width="18" style="188" customWidth="1"/>
-    <col min="9971" max="9984" width="13.7109375" style="188" customWidth="1"/>
-    <col min="9985" max="10225" width="9.140625" style="188"/>
+    <col min="9971" max="9984" width="13.7265625" style="188" customWidth="1"/>
+    <col min="9985" max="10225" width="9.1796875" style="188"/>
     <col min="10226" max="10226" width="18" style="188" customWidth="1"/>
-    <col min="10227" max="10240" width="13.7109375" style="188" customWidth="1"/>
-    <col min="10241" max="10481" width="9.140625" style="188"/>
+    <col min="10227" max="10240" width="13.7265625" style="188" customWidth="1"/>
+    <col min="10241" max="10481" width="9.1796875" style="188"/>
     <col min="10482" max="10482" width="18" style="188" customWidth="1"/>
-    <col min="10483" max="10496" width="13.7109375" style="188" customWidth="1"/>
-    <col min="10497" max="10737" width="9.140625" style="188"/>
+    <col min="10483" max="10496" width="13.7265625" style="188" customWidth="1"/>
+    <col min="10497" max="10737" width="9.1796875" style="188"/>
     <col min="10738" max="10738" width="18" style="188" customWidth="1"/>
-    <col min="10739" max="10752" width="13.7109375" style="188" customWidth="1"/>
-    <col min="10753" max="10993" width="9.140625" style="188"/>
+    <col min="10739" max="10752" width="13.7265625" style="188" customWidth="1"/>
+    <col min="10753" max="10993" width="9.1796875" style="188"/>
     <col min="10994" max="10994" width="18" style="188" customWidth="1"/>
-    <col min="10995" max="11008" width="13.7109375" style="188" customWidth="1"/>
-    <col min="11009" max="11249" width="9.140625" style="188"/>
+    <col min="10995" max="11008" width="13.7265625" style="188" customWidth="1"/>
+    <col min="11009" max="11249" width="9.1796875" style="188"/>
     <col min="11250" max="11250" width="18" style="188" customWidth="1"/>
-    <col min="11251" max="11264" width="13.7109375" style="188" customWidth="1"/>
-    <col min="11265" max="11505" width="9.140625" style="188"/>
+    <col min="11251" max="11264" width="13.7265625" style="188" customWidth="1"/>
+    <col min="11265" max="11505" width="9.1796875" style="188"/>
     <col min="11506" max="11506" width="18" style="188" customWidth="1"/>
-    <col min="11507" max="11520" width="13.7109375" style="188" customWidth="1"/>
-    <col min="11521" max="11761" width="9.140625" style="188"/>
+    <col min="11507" max="11520" width="13.7265625" style="188" customWidth="1"/>
+    <col min="11521" max="11761" width="9.1796875" style="188"/>
     <col min="11762" max="11762" width="18" style="188" customWidth="1"/>
-    <col min="11763" max="11776" width="13.7109375" style="188" customWidth="1"/>
-    <col min="11777" max="12017" width="9.140625" style="188"/>
+    <col min="11763" max="11776" width="13.7265625" style="188" customWidth="1"/>
+    <col min="11777" max="12017" width="9.1796875" style="188"/>
     <col min="12018" max="12018" width="18" style="188" customWidth="1"/>
-    <col min="12019" max="12032" width="13.7109375" style="188" customWidth="1"/>
-    <col min="12033" max="12273" width="9.140625" style="188"/>
+    <col min="12019" max="12032" width="13.7265625" style="188" customWidth="1"/>
+    <col min="12033" max="12273" width="9.1796875" style="188"/>
     <col min="12274" max="12274" width="18" style="188" customWidth="1"/>
-    <col min="12275" max="12288" width="13.7109375" style="188" customWidth="1"/>
-    <col min="12289" max="12529" width="9.140625" style="188"/>
+    <col min="12275" max="12288" width="13.7265625" style="188" customWidth="1"/>
+    <col min="12289" max="12529" width="9.1796875" style="188"/>
     <col min="12530" max="12530" width="18" style="188" customWidth="1"/>
-    <col min="12531" max="12544" width="13.7109375" style="188" customWidth="1"/>
-    <col min="12545" max="12785" width="9.140625" style="188"/>
+    <col min="12531" max="12544" width="13.7265625" style="188" customWidth="1"/>
+    <col min="12545" max="12785" width="9.1796875" style="188"/>
     <col min="12786" max="12786" width="18" style="188" customWidth="1"/>
-    <col min="12787" max="12800" width="13.7109375" style="188" customWidth="1"/>
-    <col min="12801" max="13041" width="9.140625" style="188"/>
+    <col min="12787" max="12800" width="13.7265625" style="188" customWidth="1"/>
+    <col min="12801" max="13041" width="9.1796875" style="188"/>
     <col min="13042" max="13042" width="18" style="188" customWidth="1"/>
-    <col min="13043" max="13056" width="13.7109375" style="188" customWidth="1"/>
-    <col min="13057" max="13297" width="9.140625" style="188"/>
+    <col min="13043" max="13056" width="13.7265625" style="188" customWidth="1"/>
+    <col min="13057" max="13297" width="9.1796875" style="188"/>
     <col min="13298" max="13298" width="18" style="188" customWidth="1"/>
-    <col min="13299" max="13312" width="13.7109375" style="188" customWidth="1"/>
-    <col min="13313" max="13553" width="9.140625" style="188"/>
+    <col min="13299" max="13312" width="13.7265625" style="188" customWidth="1"/>
+    <col min="13313" max="13553" width="9.1796875" style="188"/>
     <col min="13554" max="13554" width="18" style="188" customWidth="1"/>
-    <col min="13555" max="13568" width="13.7109375" style="188" customWidth="1"/>
-    <col min="13569" max="13809" width="9.140625" style="188"/>
+    <col min="13555" max="13568" width="13.7265625" style="188" customWidth="1"/>
+    <col min="13569" max="13809" width="9.1796875" style="188"/>
     <col min="13810" max="13810" width="18" style="188" customWidth="1"/>
-    <col min="13811" max="13824" width="13.7109375" style="188" customWidth="1"/>
-    <col min="13825" max="14065" width="9.140625" style="188"/>
+    <col min="13811" max="13824" width="13.7265625" style="188" customWidth="1"/>
+    <col min="13825" max="14065" width="9.1796875" style="188"/>
     <col min="14066" max="14066" width="18" style="188" customWidth="1"/>
-    <col min="14067" max="14080" width="13.7109375" style="188" customWidth="1"/>
-    <col min="14081" max="14321" width="9.140625" style="188"/>
+    <col min="14067" max="14080" width="13.7265625" style="188" customWidth="1"/>
+    <col min="14081" max="14321" width="9.1796875" style="188"/>
     <col min="14322" max="14322" width="18" style="188" customWidth="1"/>
-    <col min="14323" max="14336" width="13.7109375" style="188" customWidth="1"/>
-    <col min="14337" max="14577" width="9.140625" style="188"/>
+    <col min="14323" max="14336" width="13.7265625" style="188" customWidth="1"/>
+    <col min="14337" max="14577" width="9.1796875" style="188"/>
     <col min="14578" max="14578" width="18" style="188" customWidth="1"/>
-    <col min="14579" max="14592" width="13.7109375" style="188" customWidth="1"/>
-    <col min="14593" max="14833" width="9.140625" style="188"/>
+    <col min="14579" max="14592" width="13.7265625" style="188" customWidth="1"/>
+    <col min="14593" max="14833" width="9.1796875" style="188"/>
     <col min="14834" max="14834" width="18" style="188" customWidth="1"/>
-    <col min="14835" max="14848" width="13.7109375" style="188" customWidth="1"/>
-    <col min="14849" max="15089" width="9.140625" style="188"/>
+    <col min="14835" max="14848" width="13.7265625" style="188" customWidth="1"/>
+    <col min="14849" max="15089" width="9.1796875" style="188"/>
     <col min="15090" max="15090" width="18" style="188" customWidth="1"/>
-    <col min="15091" max="15104" width="13.7109375" style="188" customWidth="1"/>
-    <col min="15105" max="15345" width="9.140625" style="188"/>
+    <col min="15091" max="15104" width="13.7265625" style="188" customWidth="1"/>
+    <col min="15105" max="15345" width="9.1796875" style="188"/>
     <col min="15346" max="15346" width="18" style="188" customWidth="1"/>
-    <col min="15347" max="15360" width="13.7109375" style="188" customWidth="1"/>
-    <col min="15361" max="15601" width="9.140625" style="188"/>
+    <col min="15347" max="15360" width="13.7265625" style="188" customWidth="1"/>
+    <col min="15361" max="15601" width="9.1796875" style="188"/>
     <col min="15602" max="15602" width="18" style="188" customWidth="1"/>
-    <col min="15603" max="15616" width="13.7109375" style="188" customWidth="1"/>
-    <col min="15617" max="15857" width="9.140625" style="188"/>
+    <col min="15603" max="15616" width="13.7265625" style="188" customWidth="1"/>
+    <col min="15617" max="15857" width="9.1796875" style="188"/>
     <col min="15858" max="15858" width="18" style="188" customWidth="1"/>
-    <col min="15859" max="15872" width="13.7109375" style="188" customWidth="1"/>
-    <col min="15873" max="16113" width="9.140625" style="188"/>
+    <col min="15859" max="15872" width="13.7265625" style="188" customWidth="1"/>
+    <col min="15873" max="16113" width="9.1796875" style="188"/>
     <col min="16114" max="16114" width="18" style="188" customWidth="1"/>
-    <col min="16115" max="16128" width="13.7109375" style="188" customWidth="1"/>
-    <col min="16129" max="16369" width="9.140625" style="188"/>
-    <col min="16370" max="16384" width="9.140625" style="188" customWidth="1"/>
+    <col min="16115" max="16128" width="13.7265625" style="188" customWidth="1"/>
+    <col min="16129" max="16369" width="9.1796875" style="188"/>
+    <col min="16370" max="16384" width="9.1796875" style="188" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1">
-      <c r="A1" s="615" t="s">
+      <c r="A1" s="616" t="s">
         <v>445</v>
       </c>
-      <c r="B1" s="615"/>
-      <c r="C1" s="615"/>
-      <c r="D1" s="615"/>
-      <c r="E1" s="615"/>
-      <c r="F1" s="615"/>
-      <c r="G1" s="615"/>
-      <c r="H1" s="615"/>
-      <c r="I1" s="615"/>
-      <c r="J1" s="615"/>
-      <c r="K1" s="615"/>
-      <c r="L1" s="616"/>
-      <c r="M1" s="616"/>
-      <c r="N1" s="616"/>
-      <c r="O1" s="616"/>
+      <c r="B1" s="616"/>
+      <c r="C1" s="616"/>
+      <c r="D1" s="616"/>
+      <c r="E1" s="616"/>
+      <c r="F1" s="616"/>
+      <c r="G1" s="616"/>
+      <c r="H1" s="616"/>
+      <c r="I1" s="616"/>
+      <c r="J1" s="616"/>
+      <c r="K1" s="616"/>
+      <c r="L1" s="617"/>
+      <c r="M1" s="617"/>
+      <c r="N1" s="617"/>
+      <c r="O1" s="617"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1">
       <c r="A2" s="189" t="s">
@@ -27296,34 +27336,34 @@
       </c>
     </row>
     <row r="37" spans="1:15" ht="15" customHeight="1">
-      <c r="A37" s="617" t="s">
+      <c r="A37" s="618" t="s">
         <v>471</v>
       </c>
-      <c r="B37" s="617"/>
-      <c r="C37" s="617"/>
-      <c r="D37" s="617"/>
-      <c r="E37" s="617"/>
-      <c r="F37" s="617"/>
-      <c r="G37" s="617"/>
-      <c r="H37" s="617"/>
-      <c r="I37" s="617"/>
-      <c r="J37" s="617"/>
-      <c r="K37" s="617"/>
-      <c r="L37" s="617"/>
-      <c r="M37" s="617"/>
-      <c r="N37" s="617"/>
-      <c r="O37" s="617"/>
+      <c r="B37" s="618"/>
+      <c r="C37" s="618"/>
+      <c r="D37" s="618"/>
+      <c r="E37" s="618"/>
+      <c r="F37" s="618"/>
+      <c r="G37" s="618"/>
+      <c r="H37" s="618"/>
+      <c r="I37" s="618"/>
+      <c r="J37" s="618"/>
+      <c r="K37" s="618"/>
+      <c r="L37" s="618"/>
+      <c r="M37" s="618"/>
+      <c r="N37" s="618"/>
+      <c r="O37" s="618"/>
     </row>
     <row r="40" spans="1:15" ht="15" customHeight="1">
-      <c r="A40" s="615" t="s">
+      <c r="A40" s="616" t="s">
         <v>483</v>
       </c>
-      <c r="B40" s="615"/>
-      <c r="C40" s="615"/>
-      <c r="D40" s="615"/>
-      <c r="E40" s="615"/>
-      <c r="F40" s="615"/>
-      <c r="G40" s="616"/>
+      <c r="B40" s="616"/>
+      <c r="C40" s="616"/>
+      <c r="D40" s="616"/>
+      <c r="E40" s="616"/>
+      <c r="F40" s="616"/>
+      <c r="G40" s="617"/>
       <c r="H40" s="202"/>
       <c r="I40" s="202"/>
       <c r="J40" s="202"/>
@@ -27334,35 +27374,35 @@
       <c r="O40" s="202"/>
     </row>
     <row r="41" spans="1:15" ht="15" customHeight="1">
-      <c r="A41" s="618" t="s">
+      <c r="A41" s="619" t="s">
         <v>484</v>
       </c>
-      <c r="B41" s="618"/>
-      <c r="C41" s="618"/>
-      <c r="D41" s="618"/>
-      <c r="E41" s="618"/>
-      <c r="F41" s="618"/>
+      <c r="B41" s="619"/>
+      <c r="C41" s="619"/>
+      <c r="D41" s="619"/>
+      <c r="E41" s="619"/>
+      <c r="F41" s="619"/>
       <c r="G41" s="188" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="42" spans="1:15" ht="15" customHeight="1">
-      <c r="A42" s="619" t="s">
+      <c r="A42" s="620" t="s">
         <v>485</v>
       </c>
-      <c r="B42" s="621" t="s">
+      <c r="B42" s="622" t="s">
         <v>486</v>
       </c>
-      <c r="C42" s="621"/>
-      <c r="D42" s="621"/>
-      <c r="E42" s="621"/>
-      <c r="F42" s="621"/>
-      <c r="G42" s="622" t="s">
+      <c r="C42" s="622"/>
+      <c r="D42" s="622"/>
+      <c r="E42" s="622"/>
+      <c r="F42" s="622"/>
+      <c r="G42" s="623" t="s">
         <v>493</v>
       </c>
     </row>
     <row r="43" spans="1:15" ht="15" customHeight="1">
-      <c r="A43" s="620"/>
+      <c r="A43" s="621"/>
       <c r="B43" s="233" t="s">
         <v>487</v>
       </c>
@@ -27378,7 +27418,7 @@
       <c r="F43" s="233" t="s">
         <v>65</v>
       </c>
-      <c r="G43" s="623"/>
+      <c r="G43" s="624"/>
     </row>
     <row r="44" spans="1:15" ht="15" customHeight="1">
       <c r="A44" s="189" t="s">
@@ -27712,36 +27752,36 @@
       </c>
     </row>
     <row r="64" spans="1:7" ht="15" customHeight="1">
-      <c r="A64" s="612"/>
-      <c r="B64" s="610" t="s">
+      <c r="A64" s="613"/>
+      <c r="B64" s="611" t="s">
         <v>495</v>
       </c>
-      <c r="C64" s="610" t="s">
+      <c r="C64" s="611" t="s">
         <v>80</v>
       </c>
-      <c r="D64" s="614" t="s">
+      <c r="D64" s="615" t="s">
         <v>494</v>
       </c>
-      <c r="E64" s="614"/>
-      <c r="F64" s="610" t="s">
+      <c r="E64" s="615"/>
+      <c r="F64" s="611" t="s">
         <v>33</v>
       </c>
-      <c r="G64" s="610" t="s">
+      <c r="G64" s="611" t="s">
         <v>492</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="15" customHeight="1">
-      <c r="A65" s="613"/>
-      <c r="B65" s="611"/>
-      <c r="C65" s="611"/>
+      <c r="A65" s="614"/>
+      <c r="B65" s="612"/>
+      <c r="C65" s="612"/>
       <c r="D65" s="238" t="s">
         <v>33</v>
       </c>
       <c r="E65" s="63" t="s">
         <v>492</v>
       </c>
-      <c r="F65" s="611"/>
-      <c r="G65" s="611"/>
+      <c r="F65" s="612"/>
+      <c r="G65" s="612"/>
     </row>
     <row r="66" spans="1:7" ht="15" customHeight="1">
       <c r="A66" t="s">
@@ -28157,18 +28197,18 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:I40"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="170"/>
-    <col min="2" max="2" width="38.85546875" style="170" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" style="170" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="170" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" style="170" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="170"/>
-    <col min="7" max="7" width="32.28515625" style="170" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" style="170" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" style="170" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="170"/>
+    <col min="1" max="1" width="9.1796875" style="170"/>
+    <col min="2" max="2" width="38.81640625" style="170" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" style="170" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" style="170" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.26953125" style="170" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" style="170"/>
+    <col min="7" max="7" width="32.26953125" style="170" customWidth="1"/>
+    <col min="8" max="8" width="10.26953125" style="170" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7265625" style="170" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.1796875" style="170"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -28179,7 +28219,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15">
+    <row r="2" spans="1:9" ht="14.5">
       <c r="A2" s="170" t="s">
         <v>437</v>
       </c>
@@ -28187,7 +28227,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15">
+    <row r="5" spans="1:9" ht="14.5">
       <c r="B5" s="15" t="s">
         <v>410</v>
       </c>
@@ -28195,7 +28235,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15">
+    <row r="6" spans="1:9" ht="14.5">
       <c r="B6" s="172"/>
       <c r="C6" s="172" t="s">
         <v>411</v>
@@ -28268,7 +28308,7 @@
         <v>0.69119025304592319</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15">
+    <row r="9" spans="1:9" ht="14.5">
       <c r="B9" s="175" t="s">
         <v>419</v>
       </c>
@@ -28398,7 +28438,7 @@
         <v>3.0459231490159326E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15">
+    <row r="14" spans="1:9" ht="14.5">
       <c r="B14" s="175" t="s">
         <v>423</v>
       </c>
@@ -28501,7 +28541,7 @@
         <v>875.40842648323292</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="15">
+    <row r="23" spans="2:9" ht="14.5">
       <c r="B23" s="178" t="s">
         <v>424</v>
       </c>
@@ -28521,7 +28561,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="15">
+    <row r="24" spans="2:9" ht="14.5">
       <c r="B24" s="172" t="s">
         <v>427</v>
       </c>
@@ -28543,7 +28583,7 @@
         <v>0.30677290836653387</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="15">
+    <row r="25" spans="2:9" ht="14.5">
       <c r="B25" s="172" t="s">
         <v>429</v>
       </c>
@@ -28565,7 +28605,7 @@
         <v>0.26237905520774046</v>
       </c>
     </row>
-    <row r="26" spans="2:9" ht="15">
+    <row r="26" spans="2:9" ht="14.5">
       <c r="B26" s="172" t="s">
         <v>428</v>
       </c>
@@ -28587,7 +28627,7 @@
         <v>0.17586795674445077</v>
       </c>
     </row>
-    <row r="27" spans="2:9" ht="15">
+    <row r="27" spans="2:9" ht="14.5">
       <c r="B27" s="172" t="s">
         <v>430</v>
       </c>
@@ -28609,7 +28649,7 @@
         <v>0.12293682413204325</v>
       </c>
     </row>
-    <row r="28" spans="2:9" ht="15">
+    <row r="28" spans="2:9" ht="14.5">
       <c r="B28" s="172" t="s">
         <v>431</v>
       </c>
@@ -28631,7 +28671,7 @@
         <v>7.2851451337507117E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:9" ht="15">
+    <row r="29" spans="2:9" ht="14.5">
       <c r="B29" s="172" t="s">
         <v>45</v>
       </c>
@@ -28653,7 +28693,7 @@
         <v>2.8457598178713718E-2</v>
       </c>
     </row>
-    <row r="30" spans="2:9" ht="15">
+    <row r="30" spans="2:9" ht="14.5">
       <c r="B30" s="172" t="s">
         <v>433</v>
       </c>
@@ -28675,7 +28715,7 @@
         <v>2.3335230506545249E-2</v>
       </c>
     </row>
-    <row r="31" spans="2:9" ht="15">
+    <row r="31" spans="2:9" ht="14.5">
       <c r="B31" s="172" t="s">
         <v>276</v>
       </c>
@@ -28697,7 +28737,7 @@
         <v>5.6915196357427431E-3</v>
       </c>
     </row>
-    <row r="32" spans="2:9" ht="15">
+    <row r="32" spans="2:9" ht="14.5">
       <c r="B32" s="172" t="s">
         <v>65</v>
       </c>
@@ -28750,7 +28790,7 @@
       </c>
       <c r="I34" s="172"/>
     </row>
-    <row r="36" spans="2:9" ht="15">
+    <row r="36" spans="2:9" ht="14.5">
       <c r="B36" s="170" t="s">
         <v>435</v>
       </c>
@@ -28763,7 +28803,7 @@
         <v>0.55026343519494203</v>
       </c>
     </row>
-    <row r="37" spans="2:9" ht="15">
+    <row r="37" spans="2:9" ht="14.5">
       <c r="B37" s="170" t="s">
         <v>65</v>
       </c>
@@ -28776,7 +28816,7 @@
         <v>0.36501580611169654</v>
       </c>
     </row>
-    <row r="38" spans="2:9" ht="15">
+    <row r="38" spans="2:9" ht="14.5">
       <c r="B38" s="170" t="s">
         <v>45</v>
       </c>
@@ -28810,14 +28850,14 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A3:C66"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="64.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="5"/>
-    <col min="5" max="5" width="21.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="25.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="18.1796875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="64.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" style="5"/>
+    <col min="5" max="5" width="21.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:3">
@@ -28857,7 +28897,7 @@
     <row r="7" spans="1:3">
       <c r="A7" s="10"/>
     </row>
-    <row r="8" spans="1:3" ht="18.75">
+    <row r="8" spans="1:3" ht="18.5">
       <c r="A8" s="22" t="s">
         <v>98</v>
       </c>
@@ -28889,7 +28929,7 @@
       </c>
       <c r="C11" s="297"/>
     </row>
-    <row r="13" spans="1:3" ht="18.75">
+    <row r="13" spans="1:3" ht="18.5">
       <c r="A13" s="22" t="s">
         <v>99</v>
       </c>
@@ -29251,7 +29291,7 @@
       </c>
       <c r="B53" s="4"/>
     </row>
-    <row r="54" spans="1:3" ht="15.75" thickBot="1">
+    <row r="54" spans="1:3" ht="15" thickBot="1">
       <c r="A54" s="21" t="s">
         <v>106</v>
       </c>
@@ -29302,7 +29342,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="14.45" customHeight="1">
+    <row r="59" spans="1:3" ht="14.5" customHeight="1">
       <c r="A59" s="33" t="s">
         <v>110</v>
       </c>
@@ -29313,7 +29353,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="30">
+    <row r="60" spans="1:3" ht="29">
       <c r="A60" s="32"/>
       <c r="B60" s="78" t="s">
         <v>182</v>
@@ -29368,35 +29408,35 @@
     <tabColor theme="0" tint="-0.14999847407452621"/>
   </sheetPr>
   <dimension ref="A3:AD37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.1796875" customWidth="1"/>
+    <col min="2" max="2" width="11.7265625" customWidth="1"/>
+    <col min="3" max="3" width="3.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.7265625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.7265625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.5703125" customWidth="1"/>
-    <col min="25" max="25" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.54296875" customWidth="1"/>
+    <col min="25" max="25" width="6.7265625" bestFit="1" customWidth="1"/>
     <col min="26" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:30">
@@ -29867,7 +29907,7 @@
         <v>IE-MN</v>
       </c>
     </row>
-    <row r="10" spans="1:30" ht="15.75" thickBot="1">
+    <row r="10" spans="1:30" ht="15" thickBot="1">
       <c r="A10" s="92" t="s">
         <v>318</v>
       </c>
@@ -30109,7 +30149,7 @@
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>28575</xdr:colOff>
+                    <xdr:colOff>31750</xdr:colOff>
                     <xdr:row>3</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -30130,16 +30170,16 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:AR97"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="40.28515625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" style="5" customWidth="1"/>
-    <col min="4" max="44" width="12.7109375" style="106" customWidth="1"/>
-    <col min="45" max="16384" width="8.85546875" style="5"/>
+    <col min="1" max="1" width="3.453125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="40.26953125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" style="5" customWidth="1"/>
+    <col min="4" max="44" width="12.7265625" style="106" customWidth="1"/>
+    <col min="45" max="16384" width="8.81640625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" ht="23.25">
+    <row r="1" spans="1:44" ht="23.5">
       <c r="B1" s="11" t="s">
         <v>563</v>
       </c>
@@ -30195,7 +30235,7 @@
       <c r="AQ3" s="99"/>
       <c r="AR3" s="99"/>
     </row>
-    <row r="4" spans="1:44" ht="45.75" thickBot="1">
+    <row r="4" spans="1:44" ht="44" thickBot="1">
       <c r="B4" s="101"/>
       <c r="C4" s="101"/>
       <c r="D4" s="102" t="s">
@@ -30936,7 +30976,7 @@
       <c r="AQ10" s="5"/>
       <c r="AR10" s="5"/>
     </row>
-    <row r="11" spans="1:44" s="107" customFormat="1" ht="15.75" thickBot="1">
+    <row r="11" spans="1:44" s="107" customFormat="1" ht="15" thickBot="1">
       <c r="B11" s="108"/>
       <c r="C11" s="108"/>
       <c r="D11" s="109" t="str">
@@ -31436,7 +31476,7 @@
       <c r="AQ21" s="5"/>
       <c r="AR21" s="5"/>
     </row>
-    <row r="22" spans="2:44" ht="30.75" thickBot="1">
+    <row r="22" spans="2:44" ht="29.5" thickBot="1">
       <c r="B22" s="101" t="s">
         <v>378</v>
       </c>
@@ -31459,7 +31499,7 @@
       <c r="AQ22" s="5"/>
       <c r="AR22" s="5"/>
     </row>
-    <row r="23" spans="2:44" ht="15.75" thickBot="1">
+    <row r="23" spans="2:44" ht="15" thickBot="1">
       <c r="B23" s="222" t="s">
         <v>477</v>
       </c>
@@ -32396,7 +32436,7 @@
       <c r="AQ60" s="5"/>
       <c r="AR60" s="5"/>
     </row>
-    <row r="61" spans="2:44" ht="30.75" thickBot="1">
+    <row r="61" spans="2:44" ht="29.5" thickBot="1">
       <c r="B61" s="101" t="s">
         <v>378</v>
       </c>
@@ -32419,7 +32459,7 @@
       <c r="AQ61" s="5"/>
       <c r="AR61" s="5"/>
     </row>
-    <row r="62" spans="2:44" ht="15.75" thickBot="1">
+    <row r="62" spans="2:44" ht="15" thickBot="1">
       <c r="B62" s="222" t="s">
         <v>477</v>
       </c>
@@ -33193,18 +33233,18 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:N116"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" style="9" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7265625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="20.7265625" style="9" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" style="9" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="14" width="13.28515625" style="9" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="9"/>
+    <col min="4" max="4" width="13.453125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="17.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="14" width="13.26953125" style="9" customWidth="1"/>
+    <col min="15" max="16384" width="9.1796875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="23.25">
+    <row r="1" spans="1:12" ht="23.5">
       <c r="A1" s="20" t="s">
         <v>164</v>
       </c>
@@ -33215,7 +33255,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1">
+    <row r="4" spans="1:12" ht="15" thickBot="1">
       <c r="A4" s="12"/>
       <c r="B4" s="12" t="s">
         <v>42</v>
@@ -33228,7 +33268,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="17.25">
+    <row r="5" spans="1:12" ht="16.5">
       <c r="A5" s="9" t="s">
         <v>157</v>
       </c>
@@ -33242,7 +33282,7 @@
         <v>87.053206529921553</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="17.25">
+    <row r="6" spans="1:12" ht="16.5">
       <c r="A6" s="14" t="s">
         <v>158</v>
       </c>
@@ -33280,7 +33320,7 @@
       <c r="K9" s="208"/>
       <c r="L9" s="208"/>
     </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1">
+    <row r="10" spans="1:12" ht="15" thickBot="1">
       <c r="A10" s="12"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12" t="s">
@@ -33295,7 +33335,7 @@
       <c r="K10" s="208"/>
       <c r="L10" s="208"/>
     </row>
-    <row r="11" spans="1:12" ht="15.75" thickBot="1">
+    <row r="11" spans="1:12" ht="15" thickBot="1">
       <c r="A11" s="222" t="s">
         <v>152</v>
       </c>
@@ -33310,7 +33350,7 @@
       <c r="K11" s="208"/>
       <c r="L11" s="208"/>
     </row>
-    <row r="12" spans="1:12" ht="17.25">
+    <row r="12" spans="1:12" ht="16.5">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17" t="s">
@@ -33510,7 +33550,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="45.75" thickBot="1">
+    <row r="26" spans="1:12" ht="44" thickBot="1">
       <c r="A26" s="12" t="s">
         <v>378</v>
       </c>
@@ -33548,7 +33588,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="30.75" thickBot="1">
+    <row r="27" spans="1:12" ht="29.5" thickBot="1">
       <c r="A27" s="222" t="s">
         <v>477</v>
       </c>
@@ -35362,7 +35402,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="72" spans="1:12" ht="45.75" thickBot="1">
+    <row r="72" spans="1:12" ht="44" thickBot="1">
       <c r="A72" s="12" t="s">
         <v>378</v>
       </c>
@@ -35400,7 +35440,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="73" spans="1:12" ht="30.75" thickBot="1">
+    <row r="73" spans="1:12" ht="29.5" thickBot="1">
       <c r="A73" s="222" t="s">
         <v>477</v>
       </c>
@@ -35920,7 +35960,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="88" spans="1:12" ht="30.75" thickBot="1">
+    <row r="88" spans="1:12" ht="29.5" thickBot="1">
       <c r="A88" s="12" t="s">
         <v>378</v>
       </c>
@@ -35952,7 +35992,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="89" spans="1:12" ht="30.75" thickBot="1">
+    <row r="89" spans="1:12" ht="29.5" thickBot="1">
       <c r="A89" s="222" t="s">
         <v>477</v>
       </c>
@@ -36268,7 +36308,7 @@
       <c r="F99" s="71"/>
       <c r="K99" s="16"/>
     </row>
-    <row r="100" spans="1:14" ht="45.75" thickBot="1">
+    <row r="100" spans="1:14" ht="44" thickBot="1">
       <c r="A100" s="12" t="s">
         <v>378</v>
       </c>
@@ -36312,7 +36352,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="101" spans="1:14" ht="30.75" thickBot="1">
+    <row r="101" spans="1:14" ht="29.5" thickBot="1">
       <c r="A101" s="222" t="s">
         <v>477</v>
       </c>
@@ -36394,11 +36434,11 @@
         <f>Legend!$C$43</f>
         <v>SRVELC</v>
       </c>
-      <c r="F103" s="606">
+      <c r="F103" s="607">
         <f>'Public SEAI'!C29*Legend!$B$66</f>
         <v>1.4472</v>
       </c>
-      <c r="G103" s="607">
+      <c r="G103" s="608">
         <f>480000/10^6</f>
         <v>0.48</v>
       </c>
@@ -36447,8 +36487,8 @@
         <f>Legend!$C$43</f>
         <v>SRVELC</v>
       </c>
-      <c r="F104" s="606"/>
-      <c r="G104" s="607"/>
+      <c r="F104" s="607"/>
+      <c r="G104" s="608"/>
       <c r="H104" s="166">
         <v>0.15</v>
       </c>
@@ -36494,8 +36534,8 @@
         <f>Legend!$C$43</f>
         <v>SRVELC</v>
       </c>
-      <c r="F105" s="606"/>
-      <c r="G105" s="607"/>
+      <c r="F105" s="607"/>
+      <c r="G105" s="608"/>
       <c r="H105" s="166">
         <v>0.8</v>
       </c>
@@ -36541,8 +36581,8 @@
         <f>Legend!$C$43</f>
         <v>SRVELC</v>
       </c>
-      <c r="F106" s="606"/>
-      <c r="G106" s="607"/>
+      <c r="F106" s="607"/>
+      <c r="G106" s="608"/>
       <c r="H106" s="167">
         <v>0.01</v>
       </c>
@@ -36647,7 +36687,7 @@
       <c r="M110" s="43"/>
       <c r="N110"/>
     </row>
-    <row r="111" spans="1:14" ht="45.75" thickBot="1">
+    <row r="111" spans="1:14" ht="29.5" thickBot="1">
       <c r="A111" s="12" t="s">
         <v>378</v>
       </c>
@@ -36681,7 +36721,7 @@
       <c r="M111" s="43"/>
       <c r="N111"/>
     </row>
-    <row r="112" spans="1:14" ht="30.75" thickBot="1">
+    <row r="112" spans="1:14" ht="29.5" thickBot="1">
       <c r="A112" s="222" t="s">
         <v>477</v>
       </c>
@@ -36801,23 +36841,23 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:O98"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.26953125" style="9" customWidth="1"/>
     <col min="5" max="5" width="45" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.28515625" style="9" customWidth="1"/>
-    <col min="12" max="21" width="9.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7265625" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.26953125" style="9" customWidth="1"/>
+    <col min="12" max="21" width="9.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="23.25">
+    <row r="1" spans="2:10" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>84</v>
       </c>
@@ -36836,7 +36876,7 @@
       <c r="I2" s="36"/>
       <c r="J2" s="36"/>
     </row>
-    <row r="3" spans="2:10" ht="15.75" thickBot="1">
+    <row r="3" spans="2:10" ht="15" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>6</v>
       </c>
@@ -36865,7 +36905,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:10" ht="25.5">
+    <row r="4" spans="2:10" ht="26">
       <c r="B4" s="37" t="s">
         <v>114</v>
       </c>
@@ -38130,47 +38170,47 @@
   <sheetPr codeName="Sheet6">
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:Q22"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:V22"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="2" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="9"/>
-    <col min="6" max="6" width="10.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.140625" style="9"/>
-    <col min="9" max="9" width="11.7109375" style="9" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.140625" style="9" customWidth="1"/>
-    <col min="12" max="12" width="45.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="17" width="9.140625" style="9"/>
-    <col min="18" max="16384" width="9.140625" style="5"/>
+    <col min="2" max="2" width="13.26953125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="26.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" style="9"/>
+    <col min="6" max="6" width="10.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="13" width="9.1796875" style="9"/>
+    <col min="14" max="14" width="11.7265625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="12.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.1796875" style="9" customWidth="1"/>
+    <col min="17" max="17" width="45.7265625" style="9" bestFit="1" customWidth="1"/>
+    <col min="18" max="22" width="9.1796875" style="9"/>
+    <col min="23" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="23.25">
+    <row r="1" spans="2:22" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="2:17">
+    <row r="2" spans="2:22">
       <c r="B2" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="I2" s="35" t="s">
+      <c r="N2" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="35"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-    </row>
-    <row r="3" spans="2:17" ht="15.75" thickBot="1">
+      <c r="O2" s="35"/>
+      <c r="P2" s="40"/>
+      <c r="Q2" s="36"/>
+      <c r="R2" s="36"/>
+      <c r="S2" s="36"/>
+      <c r="T2" s="36"/>
+      <c r="U2" s="36"/>
+    </row>
+    <row r="3" spans="2:22" ht="15" thickBot="1">
       <c r="B3" s="21" t="str">
-        <f t="shared" ref="B3:B7" si="0">K3</f>
+        <f t="shared" ref="B3:B7" si="0">P3</f>
         <v>TechName</v>
       </c>
       <c r="C3" s="21" t="s">
@@ -38188,35 +38228,50 @@
       <c r="G3" s="21" t="s">
         <v>576</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="H3" s="603" t="s">
+        <v>624</v>
+      </c>
+      <c r="I3" s="603" t="s">
+        <v>625</v>
+      </c>
+      <c r="J3" s="603" t="s">
+        <v>626</v>
+      </c>
+      <c r="K3" s="603" t="s">
+        <v>142</v>
+      </c>
+      <c r="L3" s="603" t="s">
+        <v>627</v>
+      </c>
+      <c r="N3" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="O3" s="21" t="s">
         <v>520</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="P3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="L3" s="21" t="s">
+      <c r="Q3" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="21" t="s">
+      <c r="R3" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="21" t="s">
+      <c r="S3" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="21" t="s">
+      <c r="T3" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="P3" s="21" t="s">
+      <c r="U3" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="41" t="s">
+      <c r="V3" s="41" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="51">
+    <row r="4" spans="2:22" ht="52">
       <c r="B4" s="39" t="s">
         <v>125</v>
       </c>
@@ -38235,35 +38290,40 @@
       <c r="G4" s="37" t="s">
         <v>577</v>
       </c>
-      <c r="I4" s="37" t="s">
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="N4" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="J4" s="37" t="s">
+      <c r="O4" s="37" t="s">
         <v>534</v>
       </c>
-      <c r="K4" s="37" t="s">
+      <c r="P4" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="L4" s="37" t="s">
+      <c r="Q4" s="37" t="s">
         <v>89</v>
       </c>
-      <c r="M4" s="37" t="s">
+      <c r="R4" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="N4" s="37" t="s">
+      <c r="S4" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="O4" s="37" t="s">
+      <c r="T4" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="P4" s="39" t="s">
+      <c r="U4" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="Q4" s="39" t="s">
+      <c r="V4" s="39" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="2:17">
+    <row r="5" spans="2:22">
       <c r="B5" s="9" t="str">
         <f t="shared" si="0"/>
         <v>FT-SRVCOA</v>
@@ -38278,31 +38338,31 @@
       <c r="E5" s="9">
         <v>1</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="N5" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J5" s="36" t="str">
+      <c r="O5" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K5" s="36" t="str">
+      <c r="P5" s="36" t="str">
         <f>"FT-"&amp;D5</f>
         <v>FT-SRVCOA</v>
       </c>
-      <c r="L5" s="36" t="str">
+      <c r="Q5" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A36</f>
         <v>Fuel Tech - Solids</v>
       </c>
-      <c r="M5" s="36" t="s">
+      <c r="R5" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N5" s="36" t="s">
+      <c r="S5" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O5" s="36"/>
-      <c r="P5" s="36"/>
-    </row>
-    <row r="6" spans="2:17">
+      <c r="T5" s="36"/>
+      <c r="U5" s="36"/>
+    </row>
+    <row r="6" spans="2:22">
       <c r="B6" s="9" t="str">
         <f t="shared" si="0"/>
         <v>FT-SRVLPG</v>
@@ -38317,31 +38377,31 @@
       <c r="E6" s="9">
         <v>1</v>
       </c>
-      <c r="I6" s="36" t="s">
+      <c r="N6" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="36" t="str">
+      <c r="O6" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K6" s="36" t="str">
-        <f t="shared" ref="K6:K7" si="1">"FT-"&amp;D6</f>
+      <c r="P6" s="36" t="str">
+        <f t="shared" ref="P6:P7" si="1">"FT-"&amp;D6</f>
         <v>FT-SRVLPG</v>
       </c>
-      <c r="L6" s="36" t="str">
+      <c r="Q6" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A37</f>
         <v>Fuel Tech - LPG</v>
       </c>
-      <c r="M6" s="36" t="s">
+      <c r="R6" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N6" s="36" t="s">
+      <c r="S6" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O6" s="36"/>
-      <c r="P6" s="36"/>
-    </row>
-    <row r="7" spans="2:17">
+      <c r="T6" s="36"/>
+      <c r="U6" s="36"/>
+    </row>
+    <row r="7" spans="2:22">
       <c r="B7" s="9" t="str">
         <f t="shared" si="0"/>
         <v>FT-SRVOIL</v>
@@ -38363,31 +38423,31 @@
       <c r="G7" s="9">
         <v>5</v>
       </c>
-      <c r="I7" s="36" t="s">
+      <c r="N7" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J7" s="36" t="str">
+      <c r="O7" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K7" s="36" t="str">
+      <c r="P7" s="36" t="str">
         <f t="shared" si="1"/>
         <v>FT-SRVOIL</v>
       </c>
-      <c r="L7" s="36" t="str">
+      <c r="Q7" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A38</f>
         <v>Fuel Tech - Oil</v>
       </c>
-      <c r="M7" s="36" t="s">
+      <c r="R7" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N7" s="36" t="s">
+      <c r="S7" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O7" s="36"/>
-      <c r="P7" s="36"/>
-    </row>
-    <row r="8" spans="2:17">
+      <c r="T7" s="36"/>
+      <c r="U7" s="36"/>
+    </row>
+    <row r="8" spans="2:22">
       <c r="C8" s="9" t="s">
         <v>579</v>
       </c>
@@ -38398,31 +38458,31 @@
       <c r="G8" s="9">
         <v>5</v>
       </c>
-      <c r="I8" s="36" t="s">
+      <c r="N8" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J8" s="36" t="str">
+      <c r="O8" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K8" s="36" t="str">
-        <f t="shared" ref="K8:K13" si="2">"FT-"&amp;D10</f>
+      <c r="P8" s="36" t="str">
+        <f t="shared" ref="P8:P13" si="2">"FT-"&amp;D10</f>
         <v>FT-SRVGAS</v>
       </c>
-      <c r="L8" s="36" t="str">
+      <c r="Q8" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A39</f>
         <v>Fuel Tech - Natural Gas</v>
       </c>
-      <c r="M8" s="36" t="s">
+      <c r="R8" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N8" s="36" t="s">
+      <c r="S8" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O8" s="36"/>
-      <c r="P8" s="36"/>
-    </row>
-    <row r="9" spans="2:17">
+      <c r="T8" s="36"/>
+      <c r="U8" s="36"/>
+    </row>
+    <row r="9" spans="2:22">
       <c r="C9" s="9" t="s">
         <v>580</v>
       </c>
@@ -38433,33 +38493,33 @@
       <c r="G9" s="9">
         <v>5</v>
       </c>
-      <c r="I9" s="36" t="s">
+      <c r="N9" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="36" t="str">
+      <c r="O9" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K9" s="36" t="str">
+      <c r="P9" s="36" t="str">
         <f t="shared" si="2"/>
         <v>FT-SRVBIO</v>
       </c>
-      <c r="L9" s="36" t="str">
+      <c r="Q9" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A40</f>
         <v>Fuel Tech - Biomass</v>
       </c>
-      <c r="M9" s="36" t="s">
+      <c r="R9" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N9" s="36" t="s">
+      <c r="S9" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O9" s="36"/>
-      <c r="P9" s="36"/>
-    </row>
-    <row r="10" spans="2:17">
+      <c r="T9" s="36"/>
+      <c r="U9" s="36"/>
+    </row>
+    <row r="10" spans="2:22">
       <c r="B10" s="9" t="str">
-        <f t="shared" ref="B10:B15" si="3">K8</f>
+        <f t="shared" ref="B10:B15" si="3">P8</f>
         <v>FT-SRVGAS</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -38472,31 +38532,47 @@
       <c r="E10" s="9">
         <v>1</v>
       </c>
-      <c r="I10" s="36" t="s">
+      <c r="H10" s="9">
+        <v>50</v>
+      </c>
+      <c r="I10" s="9">
+        <f>+H10*0.05</f>
+        <v>2.5</v>
+      </c>
+      <c r="J10" s="9">
+        <v>30</v>
+      </c>
+      <c r="K10" s="9">
+        <v>0.35</v>
+      </c>
+      <c r="L10" s="9">
+        <v>31.536000000000001</v>
+      </c>
+      <c r="N10" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="36" t="str">
+      <c r="O10" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K10" s="36" t="str">
+      <c r="P10" s="36" t="str">
         <f t="shared" si="2"/>
         <v>FT-SRVBGS</v>
       </c>
-      <c r="L10" s="36" t="str">
+      <c r="Q10" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A41</f>
         <v>Fuel Tech - Biogas</v>
       </c>
-      <c r="M10" s="36" t="s">
+      <c r="R10" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N10" s="36" t="s">
+      <c r="S10" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O10" s="36"/>
-      <c r="P10" s="36"/>
-    </row>
-    <row r="11" spans="2:17">
+      <c r="T10" s="36"/>
+      <c r="U10" s="36"/>
+    </row>
+    <row r="11" spans="2:22">
       <c r="B11" s="9" t="str">
         <f t="shared" si="3"/>
         <v>FT-SRVBIO</v>
@@ -38511,31 +38587,31 @@
       <c r="E11" s="9">
         <v>1</v>
       </c>
-      <c r="I11" s="36" t="s">
+      <c r="N11" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J11" s="36" t="str">
+      <c r="O11" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K11" s="36" t="str">
+      <c r="P11" s="36" t="str">
         <f t="shared" si="2"/>
         <v>FT-SRVSOL</v>
       </c>
-      <c r="L11" s="36" t="str">
+      <c r="Q11" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A42</f>
         <v>Fuel Tech - Solar</v>
       </c>
-      <c r="M11" s="36" t="s">
+      <c r="R11" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N11" s="36" t="s">
+      <c r="S11" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O11" s="36"/>
-      <c r="P11" s="36"/>
-    </row>
-    <row r="12" spans="2:17">
+      <c r="T11" s="36"/>
+      <c r="U11" s="36"/>
+    </row>
+    <row r="12" spans="2:22">
       <c r="B12" s="9" t="str">
         <f t="shared" si="3"/>
         <v>FT-SRVBGS</v>
@@ -38550,33 +38626,33 @@
       <c r="E12" s="9">
         <v>1</v>
       </c>
-      <c r="I12" s="36" t="s">
+      <c r="N12" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J12" s="36" t="str">
+      <c r="O12" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K12" s="36" t="str">
+      <c r="P12" s="36" t="str">
         <f t="shared" si="2"/>
         <v>FT-SRVELC</v>
       </c>
-      <c r="L12" s="36" t="str">
+      <c r="Q12" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A43</f>
         <v>Fuel Tech - Electricity</v>
       </c>
-      <c r="M12" s="36" t="s">
+      <c r="R12" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N12" s="36" t="s">
+      <c r="S12" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O12" s="36" t="s">
+      <c r="T12" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="P12" s="36"/>
-    </row>
-    <row r="13" spans="2:17">
+      <c r="U12" s="36"/>
+    </row>
+    <row r="13" spans="2:22">
       <c r="B13" s="9" t="str">
         <f t="shared" si="3"/>
         <v>FT-SRVSOL</v>
@@ -38591,32 +38667,32 @@
       <c r="E13" s="9">
         <v>1</v>
       </c>
-      <c r="I13" s="46" t="s">
+      <c r="N13" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="J13" s="46" t="str">
+      <c r="O13" s="46" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K13" s="46" t="str">
+      <c r="P13" s="46" t="str">
         <f t="shared" si="2"/>
         <v>FT-SRVAHT</v>
       </c>
-      <c r="L13" s="46" t="str">
+      <c r="Q13" s="46" t="str">
         <f>"Fuel Tech - "&amp;Legend!A44</f>
         <v>Fuel Tech - Ambient Heat</v>
       </c>
-      <c r="M13" s="46" t="s">
+      <c r="R13" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="N13" s="46" t="s">
+      <c r="S13" s="46" t="s">
         <v>582</v>
       </c>
-      <c r="O13" s="46"/>
-      <c r="P13" s="46"/>
-      <c r="Q13" s="14"/>
-    </row>
-    <row r="14" spans="2:17">
+      <c r="T13" s="46"/>
+      <c r="U13" s="46"/>
+      <c r="V13" s="14"/>
+    </row>
+    <row r="14" spans="2:22">
       <c r="B14" s="9" t="str">
         <f t="shared" si="3"/>
         <v>FT-SRVELC</v>
@@ -38631,33 +38707,49 @@
       <c r="E14" s="9">
         <v>1</v>
       </c>
-      <c r="I14" s="36" t="s">
+      <c r="H14" s="9">
+        <v>200</v>
+      </c>
+      <c r="I14" s="9">
+        <f>+H14*0.05</f>
+        <v>10</v>
+      </c>
+      <c r="J14" s="9">
+        <v>50</v>
+      </c>
+      <c r="K14" s="9">
+        <v>0.35</v>
+      </c>
+      <c r="L14" s="9">
+        <v>31.536000000000001</v>
+      </c>
+      <c r="N14" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J14" s="36" t="str">
+      <c r="O14" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K14" s="36" t="str">
-        <f t="shared" ref="K14:K19" si="4">"FT-"&amp;D17</f>
+      <c r="P14" s="36" t="str">
+        <f t="shared" ref="P14:P19" si="4">"FT-"&amp;D17</f>
         <v>FT-SRVHET</v>
       </c>
-      <c r="L14" s="36" t="str">
+      <c r="Q14" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A46</f>
         <v>Fuel Tech - District heating</v>
       </c>
-      <c r="M14" s="36" t="s">
+      <c r="R14" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N14" s="36" t="s">
+      <c r="S14" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O14" s="36" t="s">
+      <c r="T14" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="P14" s="36"/>
-    </row>
-    <row r="15" spans="2:17">
+      <c r="U14" s="36"/>
+    </row>
+    <row r="15" spans="2:22">
       <c r="B15" s="9" t="str">
         <f t="shared" si="3"/>
         <v>FT-SRVAHT</v>
@@ -38672,62 +38764,62 @@
       <c r="E15" s="9">
         <v>1</v>
       </c>
-      <c r="I15" s="36" t="s">
+      <c r="N15" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J15" s="36" t="str">
+      <c r="O15" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K15" s="36" t="str">
+      <c r="P15" s="36" t="str">
         <f t="shared" si="4"/>
         <v>FT-SRVWIN</v>
       </c>
-      <c r="L15" s="36" t="str">
+      <c r="Q15" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A47</f>
         <v>Fuel Tech - Wind</v>
       </c>
-      <c r="M15" s="36" t="s">
+      <c r="R15" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N15" s="36" t="s">
+      <c r="S15" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O15" s="36"/>
-      <c r="P15" s="36"/>
-    </row>
-    <row r="16" spans="2:17">
+      <c r="T15" s="36"/>
+      <c r="U15" s="36"/>
+    </row>
+    <row r="16" spans="2:22">
       <c r="D16" s="9" t="str">
         <f>Legend!C45</f>
         <v>SRVAHT2</v>
       </c>
-      <c r="I16" s="36" t="s">
+      <c r="N16" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J16" s="36" t="str">
+      <c r="O16" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K16" s="36" t="str">
+      <c r="P16" s="36" t="str">
         <f t="shared" si="4"/>
         <v>FT-SRVH2G</v>
       </c>
-      <c r="L16" s="36" t="str">
+      <c r="Q16" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A48</f>
         <v>Fuel Tech - Hydrogen (gaseous)</v>
       </c>
-      <c r="M16" s="36" t="s">
+      <c r="R16" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N16" s="36" t="s">
+      <c r="S16" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O16" s="36"/>
-      <c r="P16" s="36"/>
-    </row>
-    <row r="17" spans="2:17">
+      <c r="T16" s="36"/>
+      <c r="U16" s="36"/>
+    </row>
+    <row r="17" spans="2:22">
       <c r="B17" s="272" t="str">
-        <f t="shared" ref="B17:B22" si="5">K14</f>
+        <f t="shared" ref="B17:B22" si="5">P14</f>
         <v>FT-SRVHET</v>
       </c>
       <c r="C17" s="272" t="s">
@@ -38742,31 +38834,47 @@
       </c>
       <c r="F17" s="272"/>
       <c r="G17" s="272"/>
-      <c r="I17" s="36" t="s">
+      <c r="H17" s="9">
+        <v>50</v>
+      </c>
+      <c r="I17" s="9">
+        <f>+H17*0.05</f>
+        <v>2.5</v>
+      </c>
+      <c r="J17" s="9">
+        <v>30</v>
+      </c>
+      <c r="K17" s="9">
+        <v>0.35</v>
+      </c>
+      <c r="L17" s="9">
+        <v>31.536000000000001</v>
+      </c>
+      <c r="N17" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J17" s="36" t="str">
+      <c r="O17" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K17" s="36" t="str">
+      <c r="P17" s="36" t="str">
         <f t="shared" si="4"/>
         <v>FT-SRVH2L</v>
       </c>
-      <c r="L17" s="36" t="str">
+      <c r="Q17" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A49</f>
         <v>Fuel Tech - Hydrogen (liquid)</v>
       </c>
-      <c r="M17" s="36" t="s">
+      <c r="R17" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N17" s="36" t="s">
+      <c r="S17" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O17" s="36"/>
-      <c r="P17" s="36"/>
-    </row>
-    <row r="18" spans="2:17">
+      <c r="T17" s="36"/>
+      <c r="U17" s="36"/>
+    </row>
+    <row r="18" spans="2:22">
       <c r="B18" s="9" t="str">
         <f t="shared" si="5"/>
         <v>FT-SRVWIN</v>
@@ -38781,31 +38889,31 @@
       <c r="E18" s="9">
         <v>1</v>
       </c>
-      <c r="I18" s="36" t="s">
+      <c r="N18" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="J18" s="36" t="str">
+      <c r="O18" s="36" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K18" s="36" t="str">
+      <c r="P18" s="36" t="str">
         <f t="shared" si="4"/>
         <v>FT-SRVBDL</v>
       </c>
-      <c r="L18" s="36" t="str">
+      <c r="Q18" s="36" t="str">
         <f>"Fuel Tech - "&amp;Legend!A50</f>
         <v>Fuel Tech - Biodiesel</v>
       </c>
-      <c r="M18" s="36" t="s">
+      <c r="R18" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="N18" s="36" t="s">
+      <c r="S18" s="36" t="s">
         <v>582</v>
       </c>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-    </row>
-    <row r="19" spans="2:17">
+      <c r="T18" s="36"/>
+      <c r="U18" s="36"/>
+    </row>
+    <row r="19" spans="2:22">
       <c r="B19" s="9" t="str">
         <f t="shared" si="5"/>
         <v>FT-SRVH2G</v>
@@ -38820,32 +38928,32 @@
       <c r="E19" s="9">
         <v>1</v>
       </c>
-      <c r="I19" s="46" t="s">
+      <c r="N19" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="J19" s="46" t="str">
+      <c r="O19" s="46" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,IF(LEFT(Regions!$C$3,1)&lt;&gt;"*",Regions!$C$3,""),IF(LEFT(Regions!$D$3,1)&lt;&gt;"*",Regions!$D$3,""))</f>
         <v>IE,National</v>
       </c>
-      <c r="K19" s="46" t="str">
+      <c r="P19" s="46" t="str">
         <f t="shared" si="4"/>
         <v>FT-SRVETH</v>
       </c>
-      <c r="L19" s="46" t="str">
+      <c r="Q19" s="46" t="str">
         <f>"Fuel Tech - "&amp;Legend!A51</f>
         <v>Fuel Tech - Ethanol</v>
       </c>
-      <c r="M19" s="46" t="s">
+      <c r="R19" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="N19" s="46" t="s">
+      <c r="S19" s="46" t="s">
         <v>582</v>
       </c>
-      <c r="O19" s="46"/>
-      <c r="P19" s="46"/>
-      <c r="Q19" s="14"/>
-    </row>
-    <row r="20" spans="2:17">
+      <c r="T19" s="46"/>
+      <c r="U19" s="46"/>
+      <c r="V19" s="14"/>
+    </row>
+    <row r="20" spans="2:22">
       <c r="B20" s="9" t="str">
         <f t="shared" si="5"/>
         <v>FT-SRVH2L</v>
@@ -38861,7 +38969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:17">
+    <row r="21" spans="2:22">
       <c r="B21" s="9" t="str">
         <f t="shared" si="5"/>
         <v>FT-SRVBDL</v>
@@ -38877,7 +38985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:17">
+    <row r="22" spans="2:22">
       <c r="B22" s="14" t="str">
         <f t="shared" si="5"/>
         <v>FT-SRVETH</v>
@@ -38907,25 +39015,25 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:T29"/>
-  <sheetFormatPr defaultColWidth="13.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="13.54296875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="19" customWidth="1"/>
+    <col min="1" max="1" width="1.7265625" style="19" customWidth="1"/>
     <col min="2" max="2" width="19" style="19" customWidth="1"/>
-    <col min="3" max="3" width="41.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="19" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" style="19" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" style="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" style="19" customWidth="1"/>
-    <col min="8" max="10" width="14.85546875" style="19" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" style="19"/>
-    <col min="12" max="13" width="13.42578125" style="19" customWidth="1"/>
-    <col min="14" max="14" width="14.42578125" style="19" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="41.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="19"/>
-    <col min="17" max="16384" width="13.5703125" style="1"/>
+    <col min="3" max="3" width="41.7265625" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="15.453125" style="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" style="19" customWidth="1"/>
+    <col min="8" max="10" width="14.81640625" style="19" customWidth="1"/>
+    <col min="11" max="11" width="13.54296875" style="19"/>
+    <col min="12" max="13" width="13.453125" style="19" customWidth="1"/>
+    <col min="14" max="14" width="14.453125" style="19" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="41.7265625" style="19" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.54296875" style="19"/>
+    <col min="17" max="16384" width="13.54296875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="23.25">
+    <row r="1" spans="1:20" ht="23.5">
       <c r="B1" s="47" t="s">
         <v>518</v>
       </c>
@@ -38948,7 +39056,7 @@
       <c r="S2" s="36"/>
       <c r="T2" s="36"/>
     </row>
-    <row r="3" spans="1:20" ht="15.75" thickBot="1">
+    <row r="3" spans="1:20" ht="15" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>4</v>
       </c>
@@ -39004,7 +39112,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="38.25">
+    <row r="4" spans="1:20" ht="39">
       <c r="B4" s="39" t="s">
         <v>125</v>
       </c>
@@ -39294,7 +39402,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="23.25">
+    <row r="14" spans="1:20" ht="23.5">
       <c r="A14" s="52"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9" t="str">
@@ -39395,7 +39503,7 @@
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
     </row>
-    <row r="23" spans="1:15" ht="23.25">
+    <row r="23" spans="1:15" ht="23.5">
       <c r="A23" s="52"/>
       <c r="B23" s="47" t="s">
         <v>519</v>
@@ -39414,7 +39522,7 @@
       <c r="F24" s="1"/>
       <c r="G24" s="9"/>
     </row>
-    <row r="25" spans="1:15" ht="15.75" thickBot="1">
+    <row r="25" spans="1:15" ht="15" thickBot="1">
       <c r="A25" s="52"/>
       <c r="B25" s="21" t="s">
         <v>520</v>
@@ -39430,7 +39538,7 @@
       </c>
       <c r="O25" s="53"/>
     </row>
-    <row r="26" spans="1:15" ht="25.5">
+    <row r="26" spans="1:15" ht="26">
       <c r="A26" s="52"/>
       <c r="B26" s="39" t="s">
         <v>606</v>
@@ -39505,29 +39613,29 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:AK57"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="2" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="24.42578125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="60.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.453125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="24.453125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="60.54296875" style="9" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="15" style="9" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" style="9" customWidth="1"/>
-    <col min="9" max="17" width="10.85546875" customWidth="1"/>
-    <col min="18" max="19" width="17.85546875" style="9" customWidth="1"/>
-    <col min="20" max="20" width="19.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.81640625" style="9" customWidth="1"/>
+    <col min="9" max="17" width="10.81640625" customWidth="1"/>
+    <col min="18" max="19" width="17.81640625" style="9" customWidth="1"/>
+    <col min="20" max="20" width="19.54296875" style="9" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="65" style="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="24" width="10.85546875" style="9" customWidth="1"/>
-    <col min="25" max="26" width="10.85546875" style="5" customWidth="1"/>
-    <col min="27" max="27" width="10.85546875" customWidth="1"/>
-    <col min="28" max="28" width="21.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="15.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="24.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="24" width="10.81640625" style="9" customWidth="1"/>
+    <col min="25" max="26" width="10.81640625" style="5" customWidth="1"/>
+    <col min="27" max="27" width="10.81640625" customWidth="1"/>
+    <col min="28" max="28" width="21.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="24.54296875" style="5" bestFit="1" customWidth="1"/>
     <col min="31" max="34" width="10" style="5" customWidth="1"/>
-    <col min="35" max="16384" width="8.85546875" style="5"/>
+    <col min="35" max="16384" width="8.81640625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="23.25">
+    <row r="1" spans="1:37" ht="23.5">
       <c r="B1" s="20" t="s">
         <v>503</v>
       </c>
@@ -39549,7 +39657,7 @@
       <c r="Y2" s="36"/>
       <c r="Z2" s="36"/>
     </row>
-    <row r="3" spans="1:37" ht="45.75" thickBot="1">
+    <row r="3" spans="1:37" ht="44" thickBot="1">
       <c r="B3" s="21" t="s">
         <v>520</v>
       </c>
@@ -39626,25 +39734,25 @@
       <c r="Z3" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="AB3" s="608" t="s">
+      <c r="AB3" s="609" t="s">
         <v>378</v>
       </c>
-      <c r="AC3" s="608" t="s">
+      <c r="AC3" s="609" t="s">
         <v>160</v>
       </c>
-      <c r="AD3" s="608" t="s">
+      <c r="AD3" s="609" t="s">
         <v>81</v>
       </c>
-      <c r="AE3" s="608" t="s">
+      <c r="AE3" s="609" t="s">
         <v>498</v>
       </c>
-      <c r="AF3" s="608" t="s">
+      <c r="AF3" s="609" t="s">
         <v>499</v>
       </c>
-      <c r="AG3" s="608" t="s">
+      <c r="AG3" s="609" t="s">
         <v>500</v>
       </c>
-      <c r="AH3" s="608" t="s">
+      <c r="AH3" s="609" t="s">
         <v>501</v>
       </c>
       <c r="AI3" s="54" t="s">
@@ -39652,7 +39760,7 @@
       </c>
       <c r="AJ3" s="55"/>
     </row>
-    <row r="4" spans="1:37" ht="60.75" thickBot="1">
+    <row r="4" spans="1:37" ht="52.5" thickBot="1">
       <c r="B4" s="39" t="s">
         <v>608</v>
       </c>
@@ -39723,13 +39831,13 @@
       <c r="Z4" s="39" t="s">
         <v>121</v>
       </c>
-      <c r="AB4" s="609"/>
-      <c r="AC4" s="609"/>
-      <c r="AD4" s="609"/>
-      <c r="AE4" s="609"/>
-      <c r="AF4" s="609"/>
-      <c r="AG4" s="609"/>
-      <c r="AH4" s="609"/>
+      <c r="AB4" s="610"/>
+      <c r="AC4" s="610"/>
+      <c r="AD4" s="610"/>
+      <c r="AE4" s="610"/>
+      <c r="AF4" s="610"/>
+      <c r="AG4" s="610"/>
+      <c r="AH4" s="610"/>
       <c r="AI4" s="13" t="s">
         <v>146</v>
       </c>
@@ -39737,7 +39845,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="5" spans="1:37">
+    <row r="5" spans="1:37" ht="15">
       <c r="B5" s="42" t="s">
         <v>131</v>
       </c>

</xml_diff>